<commit_message>
Agregué foto headmost para cascos
</commit_message>
<xml_diff>
--- a/Catalogo_Master_Lhopital-moto.xlsx
+++ b/Catalogo_Master_Lhopital-moto.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF364882-C433-4C08-BE54-6CC16AE73852}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE54178C-F5DA-48C7-8837-B50529E3286F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="705" yWindow="705" windowWidth="16200" windowHeight="9308" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LÉEME" sheetId="1" r:id="rId1"/>
@@ -23,9 +23,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Hedon Accesorios'!$A$1:$I$81</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Hedon Cascos'!$A$1:$P$151</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Hedon Cross-Sell'!$A$1:$G$35</definedName>
-    <definedName name="_xlnm._FilterDatabase">'Hedon Cross-Sell'!$A$1:$G$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Hedon Cascos'!$A$1:$Q$151</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Hedon Cross-Sell'!$A$1:$G$36</definedName>
+    <definedName name="_xlnm._FilterDatabase">'Hedon Cross-Sell'!$A$1:$G$36</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3045" uniqueCount="892">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3075" uniqueCount="898">
   <si>
     <t>CATÁLOGO MASTER v7 — Lhopital-moto</t>
   </si>
@@ -2721,6 +2721,24 @@
   </si>
   <si>
     <t>Generado: 26 de agosto 2026</t>
+  </si>
+  <si>
+    <t>heroine-racer-camelot-front-visor-cfh, heroine-racer-camelot-three-quarter-visor-cfh,heroine-racer-camelot-side-visor-cfh</t>
+  </si>
+  <si>
+    <t>heroine-racer-eemes-interior</t>
+  </si>
+  <si>
+    <t>heroine-racer-camelot-interior</t>
+  </si>
+  <si>
+    <t>Foto Headmost Cloudinary</t>
+  </si>
+  <si>
+    <t>heroine-racer-olivea-interior</t>
+  </si>
+  <si>
+    <t>heroine-racer-olivea-headmost</t>
   </si>
 </sst>
 </file>
@@ -4165,16 +4183,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:P151"/>
+  <dimension ref="A1:Q151"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.86328125" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="15.33203125" customWidth="1"/>
     <col min="4" max="4" width="26.33203125" customWidth="1"/>
     <col min="14" max="14" width="33.1328125" customWidth="1"/>
-    <col min="15" max="15" width="30" customWidth="1"/>
+    <col min="15" max="15" width="26.9296875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>42</v>
       </c>
@@ -4218,13 +4237,16 @@
         <v>55</v>
       </c>
       <c r="O1" s="1" t="s">
+        <v>895</v>
+      </c>
+      <c r="P1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>58</v>
       </c>
@@ -4261,11 +4283,11 @@
       <c r="N2" t="s">
         <v>67</v>
       </c>
-      <c r="O2" t="s">
+      <c r="P2" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>69</v>
       </c>
@@ -4302,11 +4324,11 @@
       <c r="N3" t="s">
         <v>67</v>
       </c>
-      <c r="O3" t="s">
+      <c r="P3" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>71</v>
       </c>
@@ -4343,11 +4365,11 @@
       <c r="N4" t="s">
         <v>67</v>
       </c>
-      <c r="O4" t="s">
+      <c r="P4" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>73</v>
       </c>
@@ -4384,11 +4406,11 @@
       <c r="N5" t="s">
         <v>67</v>
       </c>
-      <c r="O5" t="s">
+      <c r="P5" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>75</v>
       </c>
@@ -4425,11 +4447,11 @@
       <c r="N6" t="s">
         <v>67</v>
       </c>
-      <c r="O6" t="s">
+      <c r="P6" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>77</v>
       </c>
@@ -4466,11 +4488,11 @@
       <c r="N7" t="s">
         <v>67</v>
       </c>
-      <c r="O7" t="s">
+      <c r="P7" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>79</v>
       </c>
@@ -4510,11 +4532,11 @@
       <c r="N8" t="s">
         <v>83</v>
       </c>
-      <c r="O8" t="s">
+      <c r="P8" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>85</v>
       </c>
@@ -4554,11 +4576,11 @@
       <c r="N9" t="s">
         <v>83</v>
       </c>
-      <c r="O9" t="s">
+      <c r="P9" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>86</v>
       </c>
@@ -4598,11 +4620,11 @@
       <c r="N10" t="s">
         <v>83</v>
       </c>
-      <c r="O10" t="s">
+      <c r="P10" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>87</v>
       </c>
@@ -4642,11 +4664,11 @@
       <c r="N11" t="s">
         <v>83</v>
       </c>
-      <c r="O11" t="s">
+      <c r="P11" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>88</v>
       </c>
@@ -4686,11 +4708,11 @@
       <c r="N12" t="s">
         <v>83</v>
       </c>
-      <c r="O12" t="s">
+      <c r="P12" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>89</v>
       </c>
@@ -4730,11 +4752,11 @@
       <c r="N13" t="s">
         <v>83</v>
       </c>
-      <c r="O13" t="s">
+      <c r="P13" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>90</v>
       </c>
@@ -4775,7 +4797,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>95</v>
       </c>
@@ -4816,7 +4838,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>96</v>
       </c>
@@ -4857,7 +4879,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>98</v>
       </c>
@@ -4898,7 +4920,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>99</v>
       </c>
@@ -4939,7 +4961,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>100</v>
       </c>
@@ -4980,7 +5002,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
         <v>101</v>
       </c>
@@ -5020,11 +5042,11 @@
       <c r="N20" t="s">
         <v>105</v>
       </c>
-      <c r="O20" t="s">
+      <c r="P20" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>107</v>
       </c>
@@ -5064,11 +5086,11 @@
       <c r="N21" t="s">
         <v>105</v>
       </c>
-      <c r="O21" t="s">
+      <c r="P21" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
         <v>108</v>
       </c>
@@ -5108,11 +5130,11 @@
       <c r="N22" t="s">
         <v>105</v>
       </c>
-      <c r="O22" t="s">
+      <c r="P22" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>109</v>
       </c>
@@ -5152,11 +5174,11 @@
       <c r="N23" t="s">
         <v>105</v>
       </c>
-      <c r="O23" t="s">
+      <c r="P23" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
         <v>110</v>
       </c>
@@ -5196,11 +5218,11 @@
       <c r="N24" t="s">
         <v>105</v>
       </c>
-      <c r="O24" t="s">
+      <c r="P24" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
         <v>111</v>
       </c>
@@ -5240,11 +5262,11 @@
       <c r="N25" t="s">
         <v>105</v>
       </c>
-      <c r="O25" t="s">
+      <c r="P25" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
         <v>112</v>
       </c>
@@ -5282,7 +5304,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
         <v>118</v>
       </c>
@@ -5320,7 +5342,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
         <v>119</v>
       </c>
@@ -5358,7 +5380,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
         <v>120</v>
       </c>
@@ -5396,7 +5418,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
         <v>121</v>
       </c>
@@ -5434,7 +5456,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
         <v>122</v>
       </c>
@@ -5472,7 +5494,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
         <v>123</v>
       </c>
@@ -8014,7 +8036,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="97" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="97" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A97" t="s">
         <v>225</v>
       </c>
@@ -8052,7 +8074,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="98" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="98" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A98" t="s">
         <v>226</v>
       </c>
@@ -8090,7 +8112,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="99" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="99" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A99" t="s">
         <v>229</v>
       </c>
@@ -8128,7 +8150,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="100" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="100" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A100" t="s">
         <v>230</v>
       </c>
@@ -8166,7 +8188,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="101" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="101" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A101" t="s">
         <v>231</v>
       </c>
@@ -8204,7 +8226,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="102" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="102" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A102" t="s">
         <v>232</v>
       </c>
@@ -8242,7 +8264,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="103" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="103" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A103" t="s">
         <v>233</v>
       </c>
@@ -8280,7 +8302,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="104" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="104" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A104" t="s">
         <v>234</v>
       </c>
@@ -8317,8 +8339,14 @@
       <c r="N104" t="s">
         <v>236</v>
       </c>
-    </row>
-    <row r="105" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="O104" t="s">
+        <v>897</v>
+      </c>
+      <c r="P104" t="s">
+        <v>896</v>
+      </c>
+    </row>
+    <row r="105" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A105" t="s">
         <v>237</v>
       </c>
@@ -8355,8 +8383,14 @@
       <c r="N105" t="s">
         <v>236</v>
       </c>
-    </row>
-    <row r="106" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="O105" t="s">
+        <v>897</v>
+      </c>
+      <c r="P105" t="s">
+        <v>896</v>
+      </c>
+    </row>
+    <row r="106" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A106" t="s">
         <v>238</v>
       </c>
@@ -8393,8 +8427,14 @@
       <c r="N106" t="s">
         <v>236</v>
       </c>
-    </row>
-    <row r="107" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="O106" t="s">
+        <v>897</v>
+      </c>
+      <c r="P106" t="s">
+        <v>896</v>
+      </c>
+    </row>
+    <row r="107" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A107" t="s">
         <v>239</v>
       </c>
@@ -8431,8 +8471,14 @@
       <c r="N107" t="s">
         <v>236</v>
       </c>
-    </row>
-    <row r="108" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="O107" t="s">
+        <v>897</v>
+      </c>
+      <c r="P107" t="s">
+        <v>896</v>
+      </c>
+    </row>
+    <row r="108" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A108" t="s">
         <v>240</v>
       </c>
@@ -8469,8 +8515,14 @@
       <c r="N108" t="s">
         <v>236</v>
       </c>
-    </row>
-    <row r="109" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="O108" t="s">
+        <v>897</v>
+      </c>
+      <c r="P108" t="s">
+        <v>896</v>
+      </c>
+    </row>
+    <row r="109" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A109" t="s">
         <v>241</v>
       </c>
@@ -8507,8 +8559,14 @@
       <c r="N109" t="s">
         <v>236</v>
       </c>
-    </row>
-    <row r="110" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="O109" t="s">
+        <v>897</v>
+      </c>
+      <c r="P109" t="s">
+        <v>896</v>
+      </c>
+    </row>
+    <row r="110" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A110" t="s">
         <v>242</v>
       </c>
@@ -8549,7 +8607,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="111" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="111" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A111" t="s">
         <v>245</v>
       </c>
@@ -8590,7 +8648,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="112" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="112" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A112" t="s">
         <v>246</v>
       </c>
@@ -8631,7 +8689,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="113" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="113" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A113" t="s">
         <v>247</v>
       </c>
@@ -8672,7 +8730,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="114" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="114" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A114" t="s">
         <v>248</v>
       </c>
@@ -8713,7 +8771,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="115" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="115" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A115" t="s">
         <v>249</v>
       </c>
@@ -8754,7 +8812,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="116" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="116" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A116" t="s">
         <v>250</v>
       </c>
@@ -8792,7 +8850,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="117" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="117" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A117" t="s">
         <v>253</v>
       </c>
@@ -8830,7 +8888,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="118" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="118" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A118" t="s">
         <v>254</v>
       </c>
@@ -8868,7 +8926,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="119" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="119" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A119" t="s">
         <v>255</v>
       </c>
@@ -8906,7 +8964,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="120" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="120" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A120" t="s">
         <v>256</v>
       </c>
@@ -8944,7 +9002,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="121" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="121" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A121" t="s">
         <v>257</v>
       </c>
@@ -8982,7 +9040,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="122" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="122" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A122" t="s">
         <v>258</v>
       </c>
@@ -9023,7 +9081,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="123" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="123" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A123" t="s">
         <v>263</v>
       </c>
@@ -9064,7 +9122,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="124" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="124" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A124" t="s">
         <v>264</v>
       </c>
@@ -9105,7 +9163,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="125" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="125" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A125" t="s">
         <v>265</v>
       </c>
@@ -9146,7 +9204,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="126" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="126" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A126" t="s">
         <v>266</v>
       </c>
@@ -9187,7 +9245,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="127" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="127" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A127" t="s">
         <v>267</v>
       </c>
@@ -9228,7 +9286,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="128" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="128" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A128" t="s">
         <v>268</v>
       </c>
@@ -9265,8 +9323,11 @@
       <c r="N128" t="s">
         <v>270</v>
       </c>
-    </row>
-    <row r="129" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="P128" t="s">
+        <v>894</v>
+      </c>
+    </row>
+    <row r="129" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A129" t="s">
         <v>271</v>
       </c>
@@ -9303,8 +9364,11 @@
       <c r="N129" t="s">
         <v>270</v>
       </c>
-    </row>
-    <row r="130" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="P129" t="s">
+        <v>894</v>
+      </c>
+    </row>
+    <row r="130" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A130" t="s">
         <v>272</v>
       </c>
@@ -9341,8 +9405,11 @@
       <c r="N130" t="s">
         <v>270</v>
       </c>
-    </row>
-    <row r="131" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="P130" t="s">
+        <v>894</v>
+      </c>
+    </row>
+    <row r="131" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A131" t="s">
         <v>273</v>
       </c>
@@ -9379,8 +9446,11 @@
       <c r="N131" t="s">
         <v>270</v>
       </c>
-    </row>
-    <row r="132" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="P131" t="s">
+        <v>894</v>
+      </c>
+    </row>
+    <row r="132" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A132" t="s">
         <v>274</v>
       </c>
@@ -9417,8 +9487,11 @@
       <c r="N132" t="s">
         <v>270</v>
       </c>
-    </row>
-    <row r="133" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="P132" t="s">
+        <v>894</v>
+      </c>
+    </row>
+    <row r="133" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A133" t="s">
         <v>275</v>
       </c>
@@ -9455,8 +9528,11 @@
       <c r="N133" t="s">
         <v>270</v>
       </c>
-    </row>
-    <row r="134" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="P133" t="s">
+        <v>894</v>
+      </c>
+    </row>
+    <row r="134" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A134" t="s">
         <v>276</v>
       </c>
@@ -9497,7 +9573,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="135" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="135" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A135" t="s">
         <v>280</v>
       </c>
@@ -9538,7 +9614,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="136" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="136" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A136" t="s">
         <v>281</v>
       </c>
@@ -9579,7 +9655,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="137" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="137" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A137" t="s">
         <v>282</v>
       </c>
@@ -9620,7 +9696,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="138" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="138" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A138" t="s">
         <v>283</v>
       </c>
@@ -9661,7 +9737,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="139" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="139" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A139" t="s">
         <v>284</v>
       </c>
@@ -9702,7 +9778,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="140" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="140" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A140" t="s">
         <v>285</v>
       </c>
@@ -9739,8 +9815,11 @@
       <c r="N140" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="141" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="P140" t="s">
+        <v>893</v>
+      </c>
+    </row>
+    <row r="141" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A141" t="s">
         <v>288</v>
       </c>
@@ -9777,8 +9856,11 @@
       <c r="N141" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="142" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="P141" t="s">
+        <v>893</v>
+      </c>
+    </row>
+    <row r="142" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A142" t="s">
         <v>289</v>
       </c>
@@ -9815,8 +9897,11 @@
       <c r="N142" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="143" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="P142" t="s">
+        <v>893</v>
+      </c>
+    </row>
+    <row r="143" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A143" t="s">
         <v>290</v>
       </c>
@@ -9853,8 +9938,11 @@
       <c r="N143" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="144" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="P143" t="s">
+        <v>893</v>
+      </c>
+    </row>
+    <row r="144" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A144" t="s">
         <v>291</v>
       </c>
@@ -9891,8 +9979,11 @@
       <c r="N144" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="145" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="P144" t="s">
+        <v>893</v>
+      </c>
+    </row>
+    <row r="145" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A145" t="s">
         <v>292</v>
       </c>
@@ -9929,8 +10020,11 @@
       <c r="N145" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="146" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="P145" t="s">
+        <v>893</v>
+      </c>
+    </row>
+    <row r="146" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A146" t="s">
         <v>293</v>
       </c>
@@ -9968,7 +10062,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="147" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="147" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A147" t="s">
         <v>297</v>
       </c>
@@ -10006,7 +10100,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="148" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="148" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A148" t="s">
         <v>298</v>
       </c>
@@ -10044,7 +10138,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="149" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="149" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A149" t="s">
         <v>299</v>
       </c>
@@ -10082,7 +10176,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="150" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="150" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A150" t="s">
         <v>300</v>
       </c>
@@ -10120,7 +10214,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="151" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="151" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A151" t="s">
         <v>301</v>
       </c>
@@ -10159,7 +10253,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P151" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A1:Q151" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -12765,7 +12859,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.86328125" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="14.6640625" customWidth="1"/>
@@ -13270,37 +13364,41 @@
       </c>
       <c r="E24" s="9"/>
       <c r="F24" s="9"/>
-      <c r="G24" s="9"/>
+      <c r="G24" s="9" t="s">
+        <v>539</v>
+      </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A25" s="9" t="s">
-        <v>294</v>
+        <v>269</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="C25" s="9" t="b">
         <v>1</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>564</v>
+        <v>892</v>
       </c>
       <c r="E25" s="9"/>
       <c r="F25" s="9"/>
-      <c r="G25" s="9"/>
+      <c r="G25" s="9" t="s">
+        <v>539</v>
+      </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A26" s="9" t="s">
-        <v>286</v>
+        <v>294</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>509</v>
+        <v>503</v>
       </c>
       <c r="C26" s="9" t="b">
         <v>1</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="E26" s="9"/>
       <c r="F26" s="9"/>
@@ -13308,54 +13406,54 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A27" s="9" t="s">
-        <v>164</v>
+        <v>286</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>306</v>
+        <v>509</v>
       </c>
       <c r="C27" s="9" t="b">
         <v>1</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>883</v>
+        <v>565</v>
       </c>
       <c r="E27" s="9"/>
-      <c r="F27" s="9">
-        <v>1</v>
-      </c>
-      <c r="G27" s="9" t="s">
-        <v>539</v>
-      </c>
+      <c r="F27" s="9"/>
+      <c r="G27" s="9"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A28" s="9" t="s">
         <v>164</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="C28" s="9" t="b">
         <v>1</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>566</v>
+        <v>883</v>
       </c>
       <c r="E28" s="9"/>
-      <c r="F28" s="9"/>
-      <c r="G28" s="9"/>
+      <c r="F28" s="9">
+        <v>1</v>
+      </c>
+      <c r="G28" s="9" t="s">
+        <v>539</v>
+      </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A29" s="9" t="s">
         <v>164</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>317</v>
+        <v>311</v>
       </c>
       <c r="C29" s="9" t="b">
         <v>1</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="E29" s="9"/>
       <c r="F29" s="9"/>
@@ -13363,52 +13461,52 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A30" s="9" t="s">
-        <v>154</v>
+        <v>164</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>306</v>
+        <v>317</v>
       </c>
       <c r="C30" s="9" t="b">
         <v>1</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>884</v>
+        <v>567</v>
       </c>
       <c r="E30" s="9"/>
       <c r="F30" s="9"/>
-      <c r="G30" s="9" t="s">
-        <v>539</v>
-      </c>
+      <c r="G30" s="9"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A31" s="9" t="s">
         <v>154</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="C31" s="9" t="b">
         <v>1</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>568</v>
+        <v>884</v>
       </c>
       <c r="E31" s="9"/>
       <c r="F31" s="9"/>
-      <c r="G31" s="9"/>
+      <c r="G31" s="9" t="s">
+        <v>539</v>
+      </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A32" s="9" t="s">
         <v>154</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>317</v>
+        <v>311</v>
       </c>
       <c r="C32" s="9" t="b">
         <v>1</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="E32" s="9"/>
       <c r="F32" s="9"/>
@@ -13419,13 +13517,13 @@
         <v>154</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="C33" s="9" t="b">
         <v>1</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="E33" s="9"/>
       <c r="F33" s="9"/>
@@ -13433,35 +13531,33 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A34" s="9" t="s">
-        <v>172</v>
+        <v>154</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>306</v>
+        <v>314</v>
       </c>
       <c r="C34" s="9" t="b">
         <v>1</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>885</v>
+        <v>570</v>
       </c>
       <c r="E34" s="9"/>
       <c r="F34" s="9"/>
-      <c r="G34" s="9" t="s">
-        <v>539</v>
-      </c>
+      <c r="G34" s="9"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A35" s="9" t="s">
         <v>172</v>
       </c>
-      <c r="B35" t="s">
-        <v>314</v>
+      <c r="B35" s="9" t="s">
+        <v>306</v>
       </c>
       <c r="C35" s="9" t="b">
         <v>1</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>888</v>
+        <v>885</v>
       </c>
       <c r="E35" s="9"/>
       <c r="F35" s="9"/>
@@ -13469,14 +13565,24 @@
         <v>539</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A36" s="9"/>
-      <c r="B36" s="9"/>
-      <c r="C36" s="9"/>
-      <c r="D36" s="9"/>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A36" s="9" t="s">
+        <v>172</v>
+      </c>
+      <c r="B36" t="s">
+        <v>314</v>
+      </c>
+      <c r="C36" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="D36" s="9" t="s">
+        <v>888</v>
+      </c>
       <c r="E36" s="9"/>
       <c r="F36" s="9"/>
-      <c r="G36" s="9"/>
+      <c r="G36" s="9" t="s">
+        <v>539</v>
+      </c>
     </row>
     <row r="37" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A37" s="9"/>
@@ -13487,8 +13593,17 @@
       <c r="F37" s="9"/>
       <c r="G37" s="9"/>
     </row>
+    <row r="38" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A38" s="9"/>
+      <c r="B38" s="9"/>
+      <c r="C38" s="9"/>
+      <c r="D38" s="9"/>
+      <c r="E38" s="9"/>
+      <c r="F38" s="9"/>
+      <c r="G38" s="9"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G35" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
+  <autoFilter ref="A1:G36" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Arreglos Tienda Moto II
</commit_message>
<xml_diff>
--- a/Catalogo_Master_Lhopital-moto.xlsx
+++ b/Catalogo_Master_Lhopital-moto.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE54178C-F5DA-48C7-8837-B50529E3286F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D47B925D-4C7D-4220-ABFC-0A1C6F4F9DCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="705" yWindow="705" windowWidth="16200" windowHeight="9308" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LÉEME" sheetId="1" r:id="rId1"/>
@@ -13,13 +13,12 @@
     <sheet name="Hedon Accesorios" sheetId="3" r:id="rId3"/>
     <sheet name="Hedon Cross-Sell" sheetId="4" r:id="rId4"/>
     <sheet name="MOTO II" sheetId="5" r:id="rId5"/>
-    <sheet name="Tees" sheetId="6" r:id="rId6"/>
-    <sheet name="Colecciones" sheetId="7" r:id="rId7"/>
-    <sheet name="Lista negra" sheetId="8" r:id="rId8"/>
-    <sheet name="Contenido relacionado" sheetId="9" r:id="rId9"/>
-    <sheet name="Ventas cruzadas Moto II" sheetId="10" r:id="rId10"/>
-    <sheet name="Hoja1" sheetId="12" r:id="rId11"/>
-    <sheet name="TO-DO Anahí" sheetId="11" r:id="rId12"/>
+    <sheet name="Ventas cruzadas Moto II" sheetId="10" r:id="rId6"/>
+    <sheet name="Contenido relacionado" sheetId="9" r:id="rId7"/>
+    <sheet name="Tees" sheetId="6" r:id="rId8"/>
+    <sheet name="Colecciones" sheetId="7" r:id="rId9"/>
+    <sheet name="Lista negra" sheetId="8" r:id="rId10"/>
+    <sheet name="TO-DO Anahí" sheetId="11" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Hedon Accesorios'!$A$1:$I$81</definedName>
@@ -45,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3075" uniqueCount="898">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3032" uniqueCount="855">
   <si>
     <t>CATÁLOGO MASTER v7 — Lhopital-moto</t>
   </si>
@@ -1778,18 +1777,12 @@
     <t>en_camino</t>
   </si>
   <si>
-    <t>negro-front</t>
-  </si>
-  <si>
     <t>CHR_BLD3.0_GMG</t>
   </si>
   <si>
     <t>Beeline Moto II Metal Grey</t>
   </si>
   <si>
-    <t>gunmetal-front</t>
-  </si>
-  <si>
     <t>CHR_BLD3.0_SVR</t>
   </si>
   <si>
@@ -1799,9 +1792,6 @@
     <t>Plata</t>
   </si>
   <si>
-    <t>plata-front</t>
-  </si>
-  <si>
     <t>CHR_CSE_3.0</t>
   </si>
   <si>
@@ -1814,81 +1804,54 @@
     <t>-</t>
   </si>
   <si>
-    <t>chr-cse-30</t>
-  </si>
-  <si>
     <t>CHR_MNT3.0_BAR</t>
   </si>
   <si>
     <t>Bar Clamp Moto II</t>
   </si>
   <si>
-    <t>chr-mnt30-bar</t>
-  </si>
-  <si>
     <t>CHR_MNT3.0_MIRRORXBAR</t>
   </si>
   <si>
     <t>Mirror and Cross Bar Clamp Mount Moto II</t>
   </si>
   <si>
-    <t>chr-mnt30-mirrorxbar</t>
-  </si>
-  <si>
     <t>CHR_MNT3.0_BALL</t>
   </si>
   <si>
     <t>1" Ball Mount Adapter</t>
   </si>
   <si>
-    <t>chr-mnt30-ball</t>
-  </si>
-  <si>
     <t>CHR_MNT3.0_PWR</t>
   </si>
   <si>
     <t>Powered Mount Insert Moto II</t>
   </si>
   <si>
-    <t>chr-mnt30-pwr</t>
-  </si>
-  <si>
     <t>CHR_MNT3.0_AMPS</t>
   </si>
   <si>
     <t>MOTO II 4-hole AMPS Mount</t>
   </si>
   <si>
-    <t>chr-mnt30-amps</t>
-  </si>
-  <si>
     <t>CHR_MNT3.0_FORK</t>
   </si>
   <si>
     <t>MOTO II Fork Stem Mount</t>
   </si>
   <si>
-    <t>chr-mnt30-fork</t>
-  </si>
-  <si>
     <t>CHR_MNT3.0_MOD</t>
   </si>
   <si>
     <t>Modular Mount Extender Kit</t>
   </si>
   <si>
-    <t>chr-mnt30-mod</t>
-  </si>
-  <si>
     <t>CHR_MNT3.0_M2_M1ADAPTER</t>
   </si>
   <si>
     <t>Moto II to V1 Mount Insert Adapter</t>
   </si>
   <si>
-    <t>chr-mnt30-m2-m1adapter</t>
-  </si>
-  <si>
     <t>Diseño</t>
   </si>
   <si>
@@ -2297,9 +2260,6 @@
     <t>Cuál es mi talla</t>
   </si>
   <si>
-    <t>PENDIENTE - imagen guía cabeza</t>
-  </si>
-  <si>
     <t>Modal en selector de talla</t>
   </si>
   <si>
@@ -2354,135 +2314,6 @@
     <t>Para viajes largos: el powered mount carga tu MOTO II mientras conduces</t>
   </si>
   <si>
-    <t>Fotos en cloudinary de los 3 diferentes modelos de moto ii</t>
-  </si>
-  <si>
-    <t>motoii-svr-front-map</t>
-  </si>
-  <si>
-    <t>motoii-gmg-front-map</t>
-  </si>
-  <si>
-    <t>motoii-blk-front-map</t>
-  </si>
-  <si>
-    <t>motoii-svr-front-hour</t>
-  </si>
-  <si>
-    <t>motoii-gmg-front-hour</t>
-  </si>
-  <si>
-    <t>motoii-blk-front-hour</t>
-  </si>
-  <si>
-    <t>motoii-svr-front-logo</t>
-  </si>
-  <si>
-    <t>motoii-gmg-front-logo</t>
-  </si>
-  <si>
-    <t>motoii-blk-front-logo</t>
-  </si>
-  <si>
-    <t>motoii-svr-tq-front-map</t>
-  </si>
-  <si>
-    <t>motoii-gmg-tq-front-map</t>
-  </si>
-  <si>
-    <t>motoii-blk-tq-front-map</t>
-  </si>
-  <si>
-    <t>motoii-svr-tq-front-hour</t>
-  </si>
-  <si>
-    <t>motoii-gmg-tq-front-hour</t>
-  </si>
-  <si>
-    <t>motoii-blk-tq-front-hour</t>
-  </si>
-  <si>
-    <t>motoii-svr-tq-front-logo</t>
-  </si>
-  <si>
-    <t>motoii-gmg-tq-front-logo</t>
-  </si>
-  <si>
-    <t>motoii-blk-tq-front-logo</t>
-  </si>
-  <si>
-    <t>motoii-svr-tq-map</t>
-  </si>
-  <si>
-    <t>motoii-gmg-tq-map</t>
-  </si>
-  <si>
-    <t>motoii-blk-tq-map</t>
-  </si>
-  <si>
-    <t>motoii-svr-tq-hour</t>
-  </si>
-  <si>
-    <t>motoii-gmg-tq-hour</t>
-  </si>
-  <si>
-    <t>motoii-blk-tq-hour</t>
-  </si>
-  <si>
-    <t>motoii-svr-tq-logo</t>
-  </si>
-  <si>
-    <t>motoii-gmg-tq-logo</t>
-  </si>
-  <si>
-    <t>motoii-blk-tq-logo</t>
-  </si>
-  <si>
-    <t>motoii-svr-side</t>
-  </si>
-  <si>
-    <t>motoii-gmg-side</t>
-  </si>
-  <si>
-    <t>motoii-blk-side</t>
-  </si>
-  <si>
-    <t>motoii-svr-tq-back</t>
-  </si>
-  <si>
-    <t>motoii-gmg-tq-back</t>
-  </si>
-  <si>
-    <t>motoii-blk-tq-back</t>
-  </si>
-  <si>
-    <t>motoii-svr-tq-side</t>
-  </si>
-  <si>
-    <t>motoii-gmg-tq-side</t>
-  </si>
-  <si>
-    <t>motoii-blk-tq-side</t>
-  </si>
-  <si>
-    <t>motoii-svr-back</t>
-  </si>
-  <si>
-    <t>motoii-gmg-back</t>
-  </si>
-  <si>
-    <t>motoii-blk-back</t>
-  </si>
-  <si>
-    <t>motoii-svr-bottom</t>
-  </si>
-  <si>
-    <t>motoii-gmg-bottom</t>
-  </si>
-  <si>
-    <t>motoii-blk-bottom</t>
-  </si>
-  <si>
     <t>Pendiente</t>
   </si>
   <si>
@@ -2739,13 +2570,55 @@
   </si>
   <si>
     <t>heroine-racer-olivea-headmost</t>
+  </si>
+  <si>
+    <t>imagen hedon-tallas</t>
+  </si>
+  <si>
+    <t>chr-cse-front, chr-cse-open</t>
+  </si>
+  <si>
+    <t>chr-mnt-bar-1, chr-mnt-bar-2, chr-mnt-bar-3, chr-mnt-bar-4</t>
+  </si>
+  <si>
+    <t>chr-mnt-ball-1, chr-mnt-ball-2, chr-mnt-ball-3, chr-mnt-ball-4</t>
+  </si>
+  <si>
+    <t>chr-mnt-mirrorxbar-1, chr-mnt-mirrorxbar-2, chr-mnt-mirrorxbar-3, chr-mnt-mirrorxbar-4</t>
+  </si>
+  <si>
+    <t>chr-mnt-pwr-1, chr-mnt-pwr-2, chr-mnt-pwr-3, chr-mnt-pwr-4</t>
+  </si>
+  <si>
+    <t>chr-mnt-amps-1, mchr-mnt-amps-2, chr-mnt-amps-3, chr-mnt-amps-4</t>
+  </si>
+  <si>
+    <t>chr-mnt-fork-1, chr-mnt-fork-2, chr-mnt-fork-3, chr-mnt-fork-4, chr-mnt-fork-5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">chr-mnt-mod-1, chr-mnt-mod-2, chr-mnt-mod-3, chr-mnt-mod-4, chr-mnt-mod-5 </t>
+  </si>
+  <si>
+    <t>chr-mnt-m2-m1adapter-1, chr-mnt-m2-m1adapter-2, chr-mnt-m2-m1adapter-3</t>
+  </si>
+  <si>
+    <t>motoii-blk-front-map, motoii-blk-front-hour, motoii-blk-front-logo, motoii-blk-tq-front-map,motoii-blk-tq-front-logo, motoii-blk-tq-map, motoii-blk-side, motoii-blk-tq-back, motoii-blk-tq-side, motoii-blk-back, motoii-blk-bottom</t>
+  </si>
+  <si>
+    <t>motoii-gmg-front-map, motoii-gmg-front-hour, motoii-gmg-front-logo, motoii-gmg-tq-front-map, motoii-gmg-tq-map, motoii-gmg-side, motoii-gmg-tq-back, motoii-gmg-back, motoii-gmg-bottom</t>
+  </si>
+  <si>
+    <t>motoii-svr-front-map, motoii-svr-front-hour, motoii-svr-front-logo, motoii-svr-tq-front-map, motoii-svr-tq-front-logo, motoii-svr-tq-map, motoii-svr-side, motoii-svr-tq-back, motoii-svr-tq-side, motoii-svr-back, motoii-svr-bottom</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="44" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
+  </numFmts>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2757,6 +2630,13 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="8">
@@ -2811,10 +2691,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2833,8 +2714,13 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Moneda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -3350,7 +3236,7 @@
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A51" t="s">
-        <v>891</v>
+        <v>835</v>
       </c>
     </row>
   </sheetData>
@@ -3359,149 +3245,123 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:E8"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.86328125" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
-  <cols>
-    <col min="1" max="2" width="25.86328125" customWidth="1"/>
-    <col min="3" max="3" width="12.796875" customWidth="1"/>
-    <col min="4" max="4" width="128.796875" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
-        <v>759</v>
+        <v>683</v>
       </c>
       <c r="B1" t="s">
-        <v>760</v>
+        <v>684</v>
       </c>
       <c r="C1" t="s">
-        <v>303</v>
-      </c>
-      <c r="D1" t="s">
-        <v>761</v>
-      </c>
-      <c r="E1" t="s">
-        <v>762</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+        <v>685</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>573</v>
-      </c>
-      <c r="B2" t="s">
-        <v>590</v>
-      </c>
-      <c r="C2" t="s">
-        <v>763</v>
-      </c>
-      <c r="D2" t="s">
-        <v>764</v>
-      </c>
-      <c r="E2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>573</v>
+        <v>687</v>
       </c>
       <c r="B3" t="s">
-        <v>585</v>
+        <v>688</v>
       </c>
       <c r="C3" t="s">
-        <v>765</v>
-      </c>
-      <c r="D3" t="s">
-        <v>766</v>
-      </c>
-      <c r="E3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>573</v>
+        <v>690</v>
       </c>
       <c r="B4" t="s">
-        <v>599</v>
+        <v>688</v>
       </c>
       <c r="C4" t="s">
-        <v>767</v>
-      </c>
-      <c r="D4" t="s">
-        <v>768</v>
-      </c>
-      <c r="E4">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>578</v>
+        <v>691</v>
       </c>
       <c r="B5" t="s">
-        <v>590</v>
+        <v>688</v>
       </c>
       <c r="C5" t="s">
-        <v>763</v>
-      </c>
-      <c r="D5" t="s">
-        <v>764</v>
-      </c>
-      <c r="E5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>578</v>
+        <v>692</v>
       </c>
       <c r="B6" t="s">
-        <v>585</v>
+        <v>688</v>
       </c>
       <c r="C6" t="s">
-        <v>765</v>
-      </c>
-      <c r="D6" t="s">
-        <v>766</v>
-      </c>
-      <c r="E6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>581</v>
+        <v>693</v>
       </c>
       <c r="B7" t="s">
-        <v>590</v>
+        <v>688</v>
       </c>
       <c r="C7" t="s">
-        <v>763</v>
-      </c>
-      <c r="D7" t="s">
-        <v>764</v>
-      </c>
-      <c r="E7">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>581</v>
+        <v>694</v>
       </c>
       <c r="B8" t="s">
-        <v>585</v>
+        <v>688</v>
       </c>
       <c r="C8" t="s">
-        <v>765</v>
-      </c>
-      <c r="D8" t="s">
-        <v>766</v>
-      </c>
-      <c r="E8">
-        <v>1</v>
+        <v>689</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>695</v>
+      </c>
+      <c r="B9" t="s">
+        <v>688</v>
+      </c>
+      <c r="C9" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>696</v>
+      </c>
+      <c r="B10" t="s">
+        <v>697</v>
+      </c>
+      <c r="C10" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
+        <v>698</v>
+      </c>
+      <c r="B11" t="s">
+        <v>699</v>
+      </c>
+      <c r="C11" t="s">
+        <v>689</v>
       </c>
     </row>
   </sheetData>
@@ -3510,222 +3370,6 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:D15"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
-  <cols>
-    <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="22.1328125" customWidth="1"/>
-    <col min="4" max="4" width="21" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B1" t="s">
-        <v>769</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>770</v>
-      </c>
-      <c r="C2" t="s">
-        <v>771</v>
-      </c>
-      <c r="D2" t="s">
-        <v>772</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
-        <v>773</v>
-      </c>
-      <c r="C3" t="s">
-        <v>774</v>
-      </c>
-      <c r="D3" t="s">
-        <v>775</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>776</v>
-      </c>
-      <c r="C4" t="s">
-        <v>777</v>
-      </c>
-      <c r="D4" t="s">
-        <v>778</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s">
-        <v>779</v>
-      </c>
-      <c r="C5" t="s">
-        <v>780</v>
-      </c>
-      <c r="D5" t="s">
-        <v>781</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6" t="s">
-        <v>782</v>
-      </c>
-      <c r="C6" t="s">
-        <v>783</v>
-      </c>
-      <c r="D6" t="s">
-        <v>784</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7" t="s">
-        <v>785</v>
-      </c>
-      <c r="C7" t="s">
-        <v>786</v>
-      </c>
-      <c r="D7" t="s">
-        <v>787</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="s">
-        <v>788</v>
-      </c>
-      <c r="C8" t="s">
-        <v>789</v>
-      </c>
-      <c r="D8" t="s">
-        <v>790</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" t="s">
-        <v>791</v>
-      </c>
-      <c r="C9" t="s">
-        <v>792</v>
-      </c>
-      <c r="D9" t="s">
-        <v>793</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" t="s">
-        <v>794</v>
-      </c>
-      <c r="C10" t="s">
-        <v>795</v>
-      </c>
-      <c r="D10" t="s">
-        <v>796</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11" t="s">
-        <v>797</v>
-      </c>
-      <c r="C11" t="s">
-        <v>798</v>
-      </c>
-      <c r="D11" t="s">
-        <v>799</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12" t="s">
-        <v>800</v>
-      </c>
-      <c r="C12" t="s">
-        <v>801</v>
-      </c>
-      <c r="D12" t="s">
-        <v>802</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13" t="s">
-        <v>803</v>
-      </c>
-      <c r="C13" t="s">
-        <v>804</v>
-      </c>
-      <c r="D13" t="s">
-        <v>805</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="B14" t="s">
-        <v>806</v>
-      </c>
-      <c r="C14" t="s">
-        <v>807</v>
-      </c>
-      <c r="D14" t="s">
-        <v>808</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15">
-        <v>14</v>
-      </c>
-      <c r="B15" t="s">
-        <v>809</v>
-      </c>
-      <c r="C15" t="s">
-        <v>810</v>
-      </c>
-      <c r="D15" t="s">
-        <v>811</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.86328125" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
@@ -3739,441 +3383,441 @@
         <v>571</v>
       </c>
       <c r="B1" t="s">
-        <v>812</v>
+        <v>756</v>
       </c>
       <c r="C1" t="s">
-        <v>813</v>
+        <v>757</v>
       </c>
       <c r="D1" t="s">
-        <v>762</v>
+        <v>749</v>
       </c>
       <c r="E1" t="s">
-        <v>814</v>
+        <v>758</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A2" s="6" t="s">
-        <v>815</v>
+        <v>759</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>816</v>
+        <v>760</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>817</v>
+        <v>761</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>818</v>
+        <v>762</v>
       </c>
       <c r="E2" t="s">
-        <v>819</v>
+        <v>763</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A3" s="6" t="s">
-        <v>815</v>
+        <v>759</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>820</v>
+        <v>764</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>821</v>
+        <v>765</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>818</v>
+        <v>762</v>
       </c>
       <c r="E3" t="s">
-        <v>819</v>
+        <v>763</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
-        <v>822</v>
-      </c>
-      <c r="B4" t="s">
-        <v>823</v>
-      </c>
-      <c r="C4" t="s">
-        <v>824</v>
-      </c>
-      <c r="D4" t="s">
-        <v>818</v>
+      <c r="A4" s="6" t="s">
+        <v>766</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>767</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>768</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>762</v>
       </c>
       <c r="E4" t="s">
-        <v>819</v>
+        <v>763</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>822</v>
-      </c>
-      <c r="B5" t="s">
-        <v>825</v>
-      </c>
-      <c r="C5" t="s">
-        <v>826</v>
-      </c>
-      <c r="D5" t="s">
-        <v>827</v>
+      <c r="A5" s="6" t="s">
+        <v>766</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>769</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>770</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>771</v>
       </c>
       <c r="E5" t="s">
-        <v>819</v>
+        <v>763</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>822</v>
+        <v>766</v>
       </c>
       <c r="B6" t="s">
-        <v>828</v>
+        <v>772</v>
       </c>
       <c r="C6" t="s">
-        <v>829</v>
+        <v>773</v>
       </c>
       <c r="D6" t="s">
-        <v>818</v>
+        <v>762</v>
       </c>
       <c r="E6" t="s">
-        <v>830</v>
+        <v>774</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>822</v>
+        <v>766</v>
       </c>
       <c r="B7" t="s">
-        <v>831</v>
+        <v>775</v>
       </c>
       <c r="C7" t="s">
-        <v>832</v>
+        <v>776</v>
       </c>
       <c r="D7" t="s">
-        <v>818</v>
+        <v>762</v>
       </c>
       <c r="E7" t="s">
-        <v>819</v>
+        <v>763</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A8" s="6" t="s">
-        <v>822</v>
+        <v>766</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>833</v>
+        <v>777</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>834</v>
+        <v>778</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>818</v>
+        <v>762</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>835</v>
+        <v>779</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>822</v>
+        <v>766</v>
       </c>
       <c r="B9" t="s">
-        <v>836</v>
+        <v>780</v>
       </c>
       <c r="C9" t="s">
-        <v>837</v>
+        <v>781</v>
       </c>
       <c r="D9" t="s">
-        <v>818</v>
+        <v>762</v>
       </c>
       <c r="E9" t="s">
-        <v>812</v>
+        <v>756</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>838</v>
+        <v>782</v>
       </c>
       <c r="B10" t="s">
-        <v>839</v>
+        <v>783</v>
       </c>
       <c r="C10" t="s">
-        <v>840</v>
+        <v>784</v>
       </c>
       <c r="D10" t="s">
-        <v>827</v>
+        <v>771</v>
       </c>
       <c r="E10" t="s">
-        <v>812</v>
+        <v>756</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>841</v>
+        <v>785</v>
       </c>
       <c r="B11" t="s">
-        <v>842</v>
+        <v>786</v>
       </c>
       <c r="C11" t="s">
-        <v>843</v>
+        <v>787</v>
       </c>
       <c r="D11" t="s">
-        <v>844</v>
+        <v>788</v>
       </c>
       <c r="E11" t="s">
-        <v>845</v>
+        <v>789</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>846</v>
+        <v>790</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>847</v>
+        <v>791</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>848</v>
+        <v>792</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>818</v>
+        <v>762</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>819</v>
+        <v>763</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>849</v>
+        <v>793</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>850</v>
+        <v>794</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>851</v>
+        <v>795</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>818</v>
+        <v>762</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>819</v>
+        <v>763</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>852</v>
+        <v>796</v>
       </c>
       <c r="B14" t="s">
-        <v>853</v>
+        <v>797</v>
       </c>
       <c r="C14" t="s">
-        <v>854</v>
+        <v>798</v>
       </c>
       <c r="D14" t="s">
-        <v>827</v>
+        <v>771</v>
       </c>
       <c r="E14" t="s">
-        <v>812</v>
+        <v>756</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>852</v>
+        <v>796</v>
       </c>
       <c r="B15" t="s">
-        <v>855</v>
+        <v>799</v>
       </c>
       <c r="C15" t="s">
-        <v>856</v>
+        <v>800</v>
       </c>
       <c r="D15" t="s">
-        <v>827</v>
+        <v>771</v>
       </c>
       <c r="E15" t="s">
-        <v>812</v>
+        <v>756</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>852</v>
+        <v>796</v>
       </c>
       <c r="B16" t="s">
-        <v>857</v>
+        <v>801</v>
       </c>
       <c r="C16" t="s">
-        <v>858</v>
+        <v>802</v>
       </c>
       <c r="D16" t="s">
-        <v>818</v>
+        <v>762</v>
       </c>
       <c r="E16" t="s">
-        <v>812</v>
+        <v>756</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A17" s="6" t="s">
-        <v>859</v>
+        <v>803</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>860</v>
+        <v>804</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>861</v>
+        <v>805</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>818</v>
+        <v>762</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>819</v>
+        <v>763</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A18" s="6" t="s">
-        <v>859</v>
+        <v>803</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>862</v>
+        <v>806</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>861</v>
+        <v>805</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>827</v>
+        <v>771</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>819</v>
+        <v>763</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A19" s="6" t="s">
-        <v>863</v>
+        <v>807</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>864</v>
+        <v>808</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>865</v>
+        <v>809</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>818</v>
+        <v>762</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>819</v>
+        <v>763</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A20" s="6" t="s">
-        <v>866</v>
+        <v>810</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>867</v>
+        <v>811</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>868</v>
+        <v>812</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>827</v>
+        <v>771</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>819</v>
+        <v>763</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A21" s="6" t="s">
-        <v>866</v>
+        <v>810</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>869</v>
+        <v>813</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>870</v>
+        <v>814</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>827</v>
+        <v>771</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>819</v>
+        <v>763</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A22" s="6" t="s">
-        <v>866</v>
+        <v>810</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>871</v>
+        <v>815</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>872</v>
+        <v>816</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>827</v>
+        <v>771</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>819</v>
+        <v>763</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>866</v>
+        <v>810</v>
       </c>
       <c r="B23" t="s">
-        <v>873</v>
+        <v>817</v>
       </c>
       <c r="C23" t="s">
-        <v>874</v>
+        <v>818</v>
       </c>
       <c r="D23" t="s">
-        <v>827</v>
+        <v>771</v>
       </c>
       <c r="E23" t="s">
-        <v>812</v>
+        <v>756</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>866</v>
+        <v>810</v>
       </c>
       <c r="B24" t="s">
-        <v>875</v>
+        <v>819</v>
       </c>
       <c r="C24" t="s">
-        <v>876</v>
+        <v>820</v>
       </c>
       <c r="D24" t="s">
-        <v>827</v>
+        <v>771</v>
       </c>
       <c r="E24" t="s">
-        <v>812</v>
+        <v>756</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>866</v>
+        <v>810</v>
       </c>
       <c r="B25" t="s">
-        <v>877</v>
+        <v>821</v>
       </c>
       <c r="C25" t="s">
-        <v>878</v>
+        <v>822</v>
       </c>
       <c r="D25" t="s">
-        <v>827</v>
+        <v>771</v>
       </c>
       <c r="E25" t="s">
-        <v>812</v>
+        <v>756</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>866</v>
+        <v>810</v>
       </c>
       <c r="B26" t="s">
-        <v>879</v>
+        <v>823</v>
       </c>
       <c r="C26" t="s">
-        <v>880</v>
+        <v>824</v>
       </c>
       <c r="D26" t="s">
-        <v>881</v>
+        <v>825</v>
       </c>
       <c r="E26" t="s">
-        <v>812</v>
+        <v>756</v>
       </c>
     </row>
   </sheetData>
@@ -4237,7 +3881,7 @@
         <v>55</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>895</v>
+        <v>839</v>
       </c>
       <c r="P1" s="1" t="s">
         <v>56</v>
@@ -8340,10 +7984,10 @@
         <v>236</v>
       </c>
       <c r="O104" t="s">
-        <v>897</v>
+        <v>841</v>
       </c>
       <c r="P104" t="s">
-        <v>896</v>
+        <v>840</v>
       </c>
     </row>
     <row r="105" spans="1:16" x14ac:dyDescent="0.45">
@@ -8384,10 +8028,10 @@
         <v>236</v>
       </c>
       <c r="O105" t="s">
-        <v>897</v>
+        <v>841</v>
       </c>
       <c r="P105" t="s">
-        <v>896</v>
+        <v>840</v>
       </c>
     </row>
     <row r="106" spans="1:16" x14ac:dyDescent="0.45">
@@ -8428,10 +8072,10 @@
         <v>236</v>
       </c>
       <c r="O106" t="s">
-        <v>897</v>
+        <v>841</v>
       </c>
       <c r="P106" t="s">
-        <v>896</v>
+        <v>840</v>
       </c>
     </row>
     <row r="107" spans="1:16" x14ac:dyDescent="0.45">
@@ -8472,10 +8116,10 @@
         <v>236</v>
       </c>
       <c r="O107" t="s">
-        <v>897</v>
+        <v>841</v>
       </c>
       <c r="P107" t="s">
-        <v>896</v>
+        <v>840</v>
       </c>
     </row>
     <row r="108" spans="1:16" x14ac:dyDescent="0.45">
@@ -8516,10 +8160,10 @@
         <v>236</v>
       </c>
       <c r="O108" t="s">
-        <v>897</v>
+        <v>841</v>
       </c>
       <c r="P108" t="s">
-        <v>896</v>
+        <v>840</v>
       </c>
     </row>
     <row r="109" spans="1:16" x14ac:dyDescent="0.45">
@@ -8560,10 +8204,10 @@
         <v>236</v>
       </c>
       <c r="O109" t="s">
-        <v>897</v>
+        <v>841</v>
       </c>
       <c r="P109" t="s">
-        <v>896</v>
+        <v>840</v>
       </c>
     </row>
     <row r="110" spans="1:16" x14ac:dyDescent="0.45">
@@ -9324,7 +8968,7 @@
         <v>270</v>
       </c>
       <c r="P128" t="s">
-        <v>894</v>
+        <v>838</v>
       </c>
     </row>
     <row r="129" spans="1:16" x14ac:dyDescent="0.45">
@@ -9365,7 +9009,7 @@
         <v>270</v>
       </c>
       <c r="P129" t="s">
-        <v>894</v>
+        <v>838</v>
       </c>
     </row>
     <row r="130" spans="1:16" x14ac:dyDescent="0.45">
@@ -9406,7 +9050,7 @@
         <v>270</v>
       </c>
       <c r="P130" t="s">
-        <v>894</v>
+        <v>838</v>
       </c>
     </row>
     <row r="131" spans="1:16" x14ac:dyDescent="0.45">
@@ -9447,7 +9091,7 @@
         <v>270</v>
       </c>
       <c r="P131" t="s">
-        <v>894</v>
+        <v>838</v>
       </c>
     </row>
     <row r="132" spans="1:16" x14ac:dyDescent="0.45">
@@ -9488,7 +9132,7 @@
         <v>270</v>
       </c>
       <c r="P132" t="s">
-        <v>894</v>
+        <v>838</v>
       </c>
     </row>
     <row r="133" spans="1:16" x14ac:dyDescent="0.45">
@@ -9529,7 +9173,7 @@
         <v>270</v>
       </c>
       <c r="P133" t="s">
-        <v>894</v>
+        <v>838</v>
       </c>
     </row>
     <row r="134" spans="1:16" x14ac:dyDescent="0.45">
@@ -9816,7 +9460,7 @@
         <v>287</v>
       </c>
       <c r="P140" t="s">
-        <v>893</v>
+        <v>837</v>
       </c>
     </row>
     <row r="141" spans="1:16" x14ac:dyDescent="0.45">
@@ -9857,7 +9501,7 @@
         <v>287</v>
       </c>
       <c r="P141" t="s">
-        <v>893</v>
+        <v>837</v>
       </c>
     </row>
     <row r="142" spans="1:16" x14ac:dyDescent="0.45">
@@ -9898,7 +9542,7 @@
         <v>287</v>
       </c>
       <c r="P142" t="s">
-        <v>893</v>
+        <v>837</v>
       </c>
     </row>
     <row r="143" spans="1:16" x14ac:dyDescent="0.45">
@@ -9939,7 +9583,7 @@
         <v>287</v>
       </c>
       <c r="P143" t="s">
-        <v>893</v>
+        <v>837</v>
       </c>
     </row>
     <row r="144" spans="1:16" x14ac:dyDescent="0.45">
@@ -9980,7 +9624,7 @@
         <v>287</v>
       </c>
       <c r="P144" t="s">
-        <v>893</v>
+        <v>837</v>
       </c>
     </row>
     <row r="145" spans="1:16" x14ac:dyDescent="0.45">
@@ -10021,7 +9665,7 @@
         <v>287</v>
       </c>
       <c r="P145" t="s">
-        <v>893</v>
+        <v>837</v>
       </c>
     </row>
     <row r="146" spans="1:16" x14ac:dyDescent="0.45">
@@ -10285,7 +9929,7 @@
         <v>304</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>882</v>
+        <v>826</v>
       </c>
       <c r="E1" s="8" t="s">
         <v>305</v>
@@ -12902,7 +12546,7 @@
         <v>1</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>887</v>
+        <v>831</v>
       </c>
       <c r="E2" s="9"/>
       <c r="F2" s="9">
@@ -13066,7 +12710,7 @@
         <v>1</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>886</v>
+        <v>830</v>
       </c>
       <c r="E10" s="9"/>
       <c r="F10" s="9"/>
@@ -13190,7 +12834,7 @@
         <v>1</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>889</v>
+        <v>833</v>
       </c>
       <c r="E16" s="9"/>
       <c r="F16" s="9">
@@ -13318,7 +12962,7 @@
         <v>1</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>890</v>
+        <v>834</v>
       </c>
       <c r="E22" s="9"/>
       <c r="F22" s="9">
@@ -13379,7 +13023,7 @@
         <v>1</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>892</v>
+        <v>836</v>
       </c>
       <c r="E25" s="9"/>
       <c r="F25" s="9"/>
@@ -13432,7 +13076,7 @@
         <v>1</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>883</v>
+        <v>827</v>
       </c>
       <c r="E28" s="9"/>
       <c r="F28" s="9">
@@ -13487,7 +13131,7 @@
         <v>1</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>884</v>
+        <v>828</v>
       </c>
       <c r="E31" s="9"/>
       <c r="F31" s="9"/>
@@ -13557,7 +13201,7 @@
         <v>1</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>885</v>
+        <v>829</v>
       </c>
       <c r="E35" s="9"/>
       <c r="F35" s="9"/>
@@ -13576,7 +13220,7 @@
         <v>1</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>888</v>
+        <v>832</v>
       </c>
       <c r="E36" s="9"/>
       <c r="F36" s="9"/>
@@ -13610,8 +13254,17 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.86328125" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="26.06640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.9296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="72.06640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
@@ -13658,10 +13311,10 @@
       <c r="D2" t="s">
         <v>323</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="10">
         <v>4700</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="11">
         <v>0</v>
       </c>
       <c r="G2" t="s">
@@ -13671,26 +13324,26 @@
         <v>91952022950</v>
       </c>
       <c r="I2" t="s">
-        <v>577</v>
+        <v>852</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="B3" t="s">
         <v>574</v>
       </c>
       <c r="C3" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="D3" t="s">
         <v>369</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="10">
         <v>5299.99</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="11">
         <v>0</v>
       </c>
       <c r="G3" t="s">
@@ -13700,26 +13353,26 @@
         <v>91952022974</v>
       </c>
       <c r="I3" t="s">
-        <v>580</v>
+        <v>853</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="B4" t="s">
         <v>574</v>
       </c>
       <c r="C4" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="D4" t="s">
-        <v>583</v>
-      </c>
-      <c r="E4">
+        <v>581</v>
+      </c>
+      <c r="E4" s="10">
         <v>5299.99</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="11">
         <v>0</v>
       </c>
       <c r="G4" t="s">
@@ -13729,26 +13382,26 @@
         <v>91952022967</v>
       </c>
       <c r="I4" t="s">
-        <v>584</v>
+        <v>854</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>582</v>
+      </c>
+      <c r="B5" t="s">
+        <v>583</v>
+      </c>
+      <c r="C5" t="s">
+        <v>584</v>
+      </c>
+      <c r="D5" t="s">
         <v>585</v>
       </c>
-      <c r="B5" t="s">
-        <v>586</v>
-      </c>
-      <c r="C5" t="s">
-        <v>587</v>
-      </c>
-      <c r="D5" t="s">
-        <v>588</v>
-      </c>
-      <c r="E5">
+      <c r="E5" s="10">
         <v>450</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="11">
         <v>5</v>
       </c>
       <c r="G5" t="s">
@@ -13758,26 +13411,26 @@
         <v>91952023087</v>
       </c>
       <c r="I5" t="s">
-        <v>589</v>
+        <v>843</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>590</v>
+        <v>586</v>
       </c>
       <c r="B6" t="s">
-        <v>586</v>
+        <v>583</v>
       </c>
       <c r="C6" t="s">
-        <v>591</v>
+        <v>587</v>
       </c>
       <c r="D6" t="s">
-        <v>588</v>
-      </c>
-      <c r="E6">
+        <v>585</v>
+      </c>
+      <c r="E6" s="10">
         <v>1090</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="11">
         <v>29</v>
       </c>
       <c r="G6" t="s">
@@ -13787,26 +13440,26 @@
         <v>91952022981</v>
       </c>
       <c r="I6" t="s">
-        <v>592</v>
+        <v>844</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>593</v>
+        <v>588</v>
       </c>
       <c r="B7" t="s">
-        <v>586</v>
+        <v>583</v>
       </c>
       <c r="C7" t="s">
-        <v>594</v>
+        <v>589</v>
       </c>
       <c r="D7" t="s">
-        <v>588</v>
-      </c>
-      <c r="E7">
+        <v>585</v>
+      </c>
+      <c r="E7" s="10">
         <v>1090</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="11">
         <v>20</v>
       </c>
       <c r="G7" t="s">
@@ -13816,26 +13469,26 @@
         <v>91952023018</v>
       </c>
       <c r="I7" t="s">
-        <v>595</v>
+        <v>846</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>596</v>
+        <v>590</v>
       </c>
       <c r="B8" t="s">
-        <v>586</v>
+        <v>583</v>
       </c>
       <c r="C8" t="s">
-        <v>597</v>
+        <v>591</v>
       </c>
       <c r="D8" t="s">
-        <v>588</v>
-      </c>
-      <c r="E8">
+        <v>585</v>
+      </c>
+      <c r="E8" s="10">
         <v>600</v>
       </c>
-      <c r="F8">
+      <c r="F8" s="11">
         <v>8</v>
       </c>
       <c r="G8" t="s">
@@ -13845,26 +13498,26 @@
         <v>91952022998</v>
       </c>
       <c r="I8" t="s">
-        <v>598</v>
+        <v>845</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>599</v>
+        <v>592</v>
       </c>
       <c r="B9" t="s">
-        <v>586</v>
+        <v>583</v>
       </c>
       <c r="C9" t="s">
-        <v>600</v>
+        <v>593</v>
       </c>
       <c r="D9" t="s">
-        <v>588</v>
-      </c>
-      <c r="E9">
+        <v>585</v>
+      </c>
+      <c r="E9" s="10">
         <v>1500</v>
       </c>
-      <c r="F9">
+      <c r="F9" s="11">
         <v>11</v>
       </c>
       <c r="G9" t="s">
@@ -13874,26 +13527,26 @@
         <v>91952023094</v>
       </c>
       <c r="I9" t="s">
-        <v>601</v>
+        <v>847</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>602</v>
+        <v>594</v>
       </c>
       <c r="B10" t="s">
-        <v>586</v>
+        <v>583</v>
       </c>
       <c r="C10" t="s">
-        <v>603</v>
+        <v>595</v>
       </c>
       <c r="D10" t="s">
-        <v>588</v>
-      </c>
-      <c r="E10">
+        <v>585</v>
+      </c>
+      <c r="E10" s="10">
         <v>600</v>
       </c>
-      <c r="F10">
+      <c r="F10" s="11">
         <v>12</v>
       </c>
       <c r="G10" t="s">
@@ -13903,26 +13556,26 @@
         <v>91952023025</v>
       </c>
       <c r="I10" t="s">
-        <v>604</v>
+        <v>848</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>605</v>
+        <v>596</v>
       </c>
       <c r="B11" t="s">
-        <v>586</v>
+        <v>583</v>
       </c>
       <c r="C11" t="s">
-        <v>606</v>
+        <v>597</v>
       </c>
       <c r="D11" t="s">
-        <v>588</v>
-      </c>
-      <c r="E11">
+        <v>585</v>
+      </c>
+      <c r="E11" s="10">
         <v>1090</v>
       </c>
-      <c r="F11">
+      <c r="F11" s="11">
         <v>8</v>
       </c>
       <c r="G11" t="s">
@@ -13932,26 +13585,26 @@
         <v>91952023322</v>
       </c>
       <c r="I11" t="s">
-        <v>607</v>
+        <v>849</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>608</v>
+        <v>598</v>
       </c>
       <c r="B12" t="s">
-        <v>586</v>
+        <v>583</v>
       </c>
       <c r="C12" t="s">
-        <v>609</v>
+        <v>599</v>
       </c>
       <c r="D12" t="s">
-        <v>588</v>
-      </c>
-      <c r="E12">
+        <v>585</v>
+      </c>
+      <c r="E12" s="10">
         <v>600</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="11">
         <v>5</v>
       </c>
       <c r="G12" t="s">
@@ -13961,26 +13614,26 @@
         <v>91952023339</v>
       </c>
       <c r="I12" t="s">
-        <v>610</v>
+        <v>850</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>611</v>
+        <v>600</v>
       </c>
       <c r="B13" t="s">
-        <v>586</v>
+        <v>583</v>
       </c>
       <c r="C13" t="s">
-        <v>612</v>
+        <v>601</v>
       </c>
       <c r="D13" t="s">
-        <v>588</v>
-      </c>
-      <c r="E13">
+        <v>585</v>
+      </c>
+      <c r="E13" s="10">
         <v>220</v>
       </c>
-      <c r="F13">
+      <c r="F13" s="11">
         <v>29</v>
       </c>
       <c r="G13" t="s">
@@ -13990,8 +13643,14 @@
         <v>91952023032</v>
       </c>
       <c r="I13" t="s">
-        <v>613</v>
-      </c>
+        <v>851</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E14" s="10"/>
+    </row>
+    <row r="15" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E15" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -13999,6 +13658,393 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.86328125" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="2" width="25.86328125" customWidth="1"/>
+    <col min="3" max="3" width="12.796875" customWidth="1"/>
+    <col min="4" max="4" width="128.796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>746</v>
+      </c>
+      <c r="B1" t="s">
+        <v>747</v>
+      </c>
+      <c r="C1" t="s">
+        <v>303</v>
+      </c>
+      <c r="D1" t="s">
+        <v>748</v>
+      </c>
+      <c r="E1" t="s">
+        <v>749</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>573</v>
+      </c>
+      <c r="B2" t="s">
+        <v>586</v>
+      </c>
+      <c r="C2" t="s">
+        <v>750</v>
+      </c>
+      <c r="D2" t="s">
+        <v>751</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>573</v>
+      </c>
+      <c r="B3" t="s">
+        <v>582</v>
+      </c>
+      <c r="C3" t="s">
+        <v>752</v>
+      </c>
+      <c r="D3" t="s">
+        <v>753</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>573</v>
+      </c>
+      <c r="B4" t="s">
+        <v>592</v>
+      </c>
+      <c r="C4" t="s">
+        <v>754</v>
+      </c>
+      <c r="D4" t="s">
+        <v>755</v>
+      </c>
+      <c r="E4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>577</v>
+      </c>
+      <c r="B5" t="s">
+        <v>586</v>
+      </c>
+      <c r="C5" t="s">
+        <v>750</v>
+      </c>
+      <c r="D5" t="s">
+        <v>751</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>577</v>
+      </c>
+      <c r="B6" t="s">
+        <v>582</v>
+      </c>
+      <c r="C6" t="s">
+        <v>752</v>
+      </c>
+      <c r="D6" t="s">
+        <v>753</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>579</v>
+      </c>
+      <c r="B7" t="s">
+        <v>586</v>
+      </c>
+      <c r="C7" t="s">
+        <v>750</v>
+      </c>
+      <c r="D7" t="s">
+        <v>751</v>
+      </c>
+      <c r="E7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>579</v>
+      </c>
+      <c r="B8" t="s">
+        <v>582</v>
+      </c>
+      <c r="C8" t="s">
+        <v>752</v>
+      </c>
+      <c r="D8" t="s">
+        <v>753</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.86328125" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="2" max="2" width="14.86328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.06640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="81.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A1" t="s">
+        <v>700</v>
+      </c>
+      <c r="B1" t="s">
+        <v>701</v>
+      </c>
+      <c r="C1" t="s">
+        <v>702</v>
+      </c>
+      <c r="D1" t="s">
+        <v>703</v>
+      </c>
+      <c r="E1" t="s">
+        <v>704</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>705</v>
+      </c>
+      <c r="B2" t="s">
+        <v>706</v>
+      </c>
+      <c r="C2" t="s">
+        <v>707</v>
+      </c>
+      <c r="D2" t="s">
+        <v>708</v>
+      </c>
+      <c r="E2" t="s">
+        <v>709</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>705</v>
+      </c>
+      <c r="B3" t="s">
+        <v>710</v>
+      </c>
+      <c r="C3" t="s">
+        <v>711</v>
+      </c>
+      <c r="D3" t="s">
+        <v>712</v>
+      </c>
+      <c r="E3" t="s">
+        <v>713</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>705</v>
+      </c>
+      <c r="B4" t="s">
+        <v>710</v>
+      </c>
+      <c r="C4" t="s">
+        <v>714</v>
+      </c>
+      <c r="D4" t="s">
+        <v>715</v>
+      </c>
+      <c r="E4" t="s">
+        <v>716</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>705</v>
+      </c>
+      <c r="B5" t="s">
+        <v>717</v>
+      </c>
+      <c r="C5" t="s">
+        <v>718</v>
+      </c>
+      <c r="D5" t="s">
+        <v>719</v>
+      </c>
+      <c r="E5" t="s">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>721</v>
+      </c>
+      <c r="B6" t="s">
+        <v>722</v>
+      </c>
+      <c r="C6" t="s">
+        <v>723</v>
+      </c>
+      <c r="D6" t="s">
+        <v>724</v>
+      </c>
+      <c r="E6" t="s">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>721</v>
+      </c>
+      <c r="B7" t="s">
+        <v>722</v>
+      </c>
+      <c r="C7" t="s">
+        <v>726</v>
+      </c>
+      <c r="D7" t="s">
+        <v>727</v>
+      </c>
+      <c r="E7" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>721</v>
+      </c>
+      <c r="B8" t="s">
+        <v>729</v>
+      </c>
+      <c r="C8" t="s">
+        <v>730</v>
+      </c>
+      <c r="D8" t="s">
+        <v>731</v>
+      </c>
+      <c r="E8" t="s">
+        <v>732</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>721</v>
+      </c>
+      <c r="B9" t="s">
+        <v>729</v>
+      </c>
+      <c r="C9" t="s">
+        <v>733</v>
+      </c>
+      <c r="D9" t="s">
+        <v>734</v>
+      </c>
+      <c r="E9" t="s">
+        <v>732</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>735</v>
+      </c>
+      <c r="B10" t="s">
+        <v>736</v>
+      </c>
+      <c r="C10" t="s">
+        <v>737</v>
+      </c>
+      <c r="D10" t="s">
+        <v>842</v>
+      </c>
+      <c r="E10" t="s">
+        <v>738</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
+        <v>735</v>
+      </c>
+      <c r="B11" t="s">
+        <v>739</v>
+      </c>
+      <c r="C11" t="s">
+        <v>740</v>
+      </c>
+      <c r="D11" t="s">
+        <v>741</v>
+      </c>
+      <c r="E11" t="s">
+        <v>742</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
+        <v>735</v>
+      </c>
+      <c r="B12" t="s">
+        <v>739</v>
+      </c>
+      <c r="C12" t="s">
+        <v>127</v>
+      </c>
+      <c r="D12" t="s">
+        <v>741</v>
+      </c>
+      <c r="E12" t="s">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A13" t="s">
+        <v>735</v>
+      </c>
+      <c r="B13" t="s">
+        <v>739</v>
+      </c>
+      <c r="C13" t="s">
+        <v>744</v>
+      </c>
+      <c r="D13" t="s">
+        <v>741</v>
+      </c>
+      <c r="E13" t="s">
+        <v>745</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.86328125" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
@@ -14015,7 +14061,7 @@
         <v>43</v>
       </c>
       <c r="C1" t="s">
-        <v>614</v>
+        <v>602</v>
       </c>
       <c r="D1" t="s">
         <v>45</v>
@@ -14033,7 +14079,7 @@
         <v>49</v>
       </c>
       <c r="I1" t="s">
-        <v>615</v>
+        <v>603</v>
       </c>
       <c r="J1" t="s">
         <v>55</v>
@@ -14044,13 +14090,13 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>616</v>
+        <v>604</v>
       </c>
       <c r="B2" t="s">
-        <v>617</v>
+        <v>605</v>
       </c>
       <c r="C2" t="s">
-        <v>618</v>
+        <v>606</v>
       </c>
       <c r="D2" t="s">
         <v>323</v>
@@ -14068,21 +14114,21 @@
         <v>97</v>
       </c>
       <c r="I2" t="s">
-        <v>619</v>
+        <v>607</v>
       </c>
       <c r="J2" t="s">
-        <v>620</v>
+        <v>608</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>621</v>
+        <v>609</v>
       </c>
       <c r="B3" t="s">
-        <v>617</v>
+        <v>605</v>
       </c>
       <c r="C3" t="s">
-        <v>618</v>
+        <v>606</v>
       </c>
       <c r="D3" t="s">
         <v>323</v>
@@ -14100,21 +14146,21 @@
         <v>97</v>
       </c>
       <c r="I3" t="s">
-        <v>619</v>
+        <v>607</v>
       </c>
       <c r="J3" t="s">
-        <v>622</v>
+        <v>610</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>623</v>
+        <v>611</v>
       </c>
       <c r="B4" t="s">
-        <v>617</v>
+        <v>605</v>
       </c>
       <c r="C4" t="s">
-        <v>618</v>
+        <v>606</v>
       </c>
       <c r="D4" t="s">
         <v>323</v>
@@ -14132,21 +14178,21 @@
         <v>97</v>
       </c>
       <c r="I4" t="s">
-        <v>619</v>
+        <v>607</v>
       </c>
       <c r="J4" t="s">
-        <v>624</v>
+        <v>612</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>625</v>
+        <v>613</v>
       </c>
       <c r="B5" t="s">
-        <v>617</v>
+        <v>605</v>
       </c>
       <c r="C5" t="s">
-        <v>618</v>
+        <v>606</v>
       </c>
       <c r="D5" t="s">
         <v>323</v>
@@ -14164,21 +14210,21 @@
         <v>97</v>
       </c>
       <c r="I5" t="s">
-        <v>619</v>
+        <v>607</v>
       </c>
       <c r="J5" t="s">
-        <v>624</v>
+        <v>612</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>626</v>
+        <v>614</v>
       </c>
       <c r="B6" t="s">
-        <v>627</v>
+        <v>615</v>
       </c>
       <c r="C6" t="s">
-        <v>628</v>
+        <v>616</v>
       </c>
       <c r="D6" t="s">
         <v>323</v>
@@ -14196,21 +14242,21 @@
         <v>97</v>
       </c>
       <c r="I6" t="s">
-        <v>619</v>
+        <v>607</v>
       </c>
       <c r="J6" t="s">
-        <v>629</v>
+        <v>617</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>630</v>
+        <v>618</v>
       </c>
       <c r="B7" t="s">
-        <v>627</v>
+        <v>615</v>
       </c>
       <c r="C7" t="s">
-        <v>628</v>
+        <v>616</v>
       </c>
       <c r="D7" t="s">
         <v>323</v>
@@ -14228,21 +14274,21 @@
         <v>97</v>
       </c>
       <c r="I7" t="s">
+        <v>607</v>
+      </c>
+      <c r="J7" t="s">
         <v>619</v>
-      </c>
-      <c r="J7" t="s">
-        <v>631</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>632</v>
+        <v>620</v>
       </c>
       <c r="B8" t="s">
-        <v>627</v>
+        <v>615</v>
       </c>
       <c r="C8" t="s">
-        <v>628</v>
+        <v>616</v>
       </c>
       <c r="D8" t="s">
         <v>323</v>
@@ -14260,21 +14306,21 @@
         <v>97</v>
       </c>
       <c r="I8" t="s">
-        <v>619</v>
+        <v>607</v>
       </c>
       <c r="J8" t="s">
-        <v>633</v>
+        <v>621</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>634</v>
+        <v>622</v>
       </c>
       <c r="B9" t="s">
-        <v>627</v>
+        <v>615</v>
       </c>
       <c r="C9" t="s">
-        <v>628</v>
+        <v>616</v>
       </c>
       <c r="D9" t="s">
         <v>323</v>
@@ -14292,21 +14338,21 @@
         <v>97</v>
       </c>
       <c r="I9" t="s">
-        <v>619</v>
+        <v>607</v>
       </c>
       <c r="J9" t="s">
-        <v>633</v>
+        <v>621</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>635</v>
+        <v>623</v>
       </c>
       <c r="B10" t="s">
-        <v>636</v>
+        <v>624</v>
       </c>
       <c r="C10" t="s">
-        <v>637</v>
+        <v>625</v>
       </c>
       <c r="D10" t="s">
         <v>323</v>
@@ -14324,21 +14370,21 @@
         <v>97</v>
       </c>
       <c r="I10" t="s">
-        <v>619</v>
+        <v>607</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>638</v>
+        <v>626</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="16.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>639</v>
+        <v>627</v>
       </c>
       <c r="B11" t="s">
-        <v>636</v>
+        <v>624</v>
       </c>
       <c r="C11" t="s">
-        <v>637</v>
+        <v>625</v>
       </c>
       <c r="D11" t="s">
         <v>323</v>
@@ -14356,21 +14402,21 @@
         <v>97</v>
       </c>
       <c r="I11" t="s">
-        <v>619</v>
+        <v>607</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>640</v>
+        <v>628</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>641</v>
+        <v>629</v>
       </c>
       <c r="B12" t="s">
-        <v>636</v>
+        <v>624</v>
       </c>
       <c r="C12" t="s">
-        <v>637</v>
+        <v>625</v>
       </c>
       <c r="D12" t="s">
         <v>323</v>
@@ -14388,21 +14434,21 @@
         <v>97</v>
       </c>
       <c r="I12" t="s">
-        <v>619</v>
+        <v>607</v>
       </c>
       <c r="J12" t="s">
-        <v>642</v>
+        <v>630</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>643</v>
+        <v>631</v>
       </c>
       <c r="B13" t="s">
-        <v>636</v>
+        <v>624</v>
       </c>
       <c r="C13" t="s">
-        <v>637</v>
+        <v>625</v>
       </c>
       <c r="D13" t="s">
         <v>323</v>
@@ -14420,21 +14466,21 @@
         <v>97</v>
       </c>
       <c r="I13" t="s">
-        <v>619</v>
+        <v>607</v>
       </c>
       <c r="J13" t="s">
-        <v>642</v>
+        <v>630</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>644</v>
+        <v>632</v>
       </c>
       <c r="B14" t="s">
-        <v>645</v>
+        <v>633</v>
       </c>
       <c r="C14" t="s">
-        <v>646</v>
+        <v>634</v>
       </c>
       <c r="D14" t="s">
         <v>323</v>
@@ -14452,21 +14498,21 @@
         <v>97</v>
       </c>
       <c r="I14" t="s">
-        <v>619</v>
+        <v>607</v>
       </c>
       <c r="J14" t="s">
-        <v>647</v>
+        <v>635</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>648</v>
+        <v>636</v>
       </c>
       <c r="B15" t="s">
-        <v>645</v>
+        <v>633</v>
       </c>
       <c r="C15" t="s">
-        <v>646</v>
+        <v>634</v>
       </c>
       <c r="D15" t="s">
         <v>323</v>
@@ -14484,21 +14530,21 @@
         <v>97</v>
       </c>
       <c r="I15" t="s">
-        <v>619</v>
+        <v>607</v>
       </c>
       <c r="J15" t="s">
-        <v>649</v>
+        <v>637</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>650</v>
+        <v>638</v>
       </c>
       <c r="B16" t="s">
-        <v>645</v>
+        <v>633</v>
       </c>
       <c r="C16" t="s">
-        <v>646</v>
+        <v>634</v>
       </c>
       <c r="D16" t="s">
         <v>323</v>
@@ -14516,21 +14562,21 @@
         <v>97</v>
       </c>
       <c r="I16" t="s">
-        <v>619</v>
+        <v>607</v>
       </c>
       <c r="J16" t="s">
-        <v>651</v>
+        <v>639</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>652</v>
+        <v>640</v>
       </c>
       <c r="B17" t="s">
-        <v>645</v>
+        <v>633</v>
       </c>
       <c r="C17" t="s">
-        <v>646</v>
+        <v>634</v>
       </c>
       <c r="D17" t="s">
         <v>323</v>
@@ -14548,21 +14594,21 @@
         <v>97</v>
       </c>
       <c r="I17" t="s">
-        <v>619</v>
+        <v>607</v>
       </c>
       <c r="J17" t="s">
-        <v>651</v>
+        <v>639</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
-        <v>653</v>
+        <v>641</v>
       </c>
       <c r="B18" t="s">
-        <v>654</v>
+        <v>642</v>
       </c>
       <c r="C18" t="s">
-        <v>655</v>
+        <v>643</v>
       </c>
       <c r="D18" t="s">
         <v>323</v>
@@ -14580,21 +14626,21 @@
         <v>97</v>
       </c>
       <c r="I18" t="s">
-        <v>619</v>
+        <v>607</v>
       </c>
       <c r="J18" t="s">
-        <v>656</v>
+        <v>644</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
-        <v>657</v>
+        <v>645</v>
       </c>
       <c r="B19" t="s">
-        <v>654</v>
+        <v>642</v>
       </c>
       <c r="C19" t="s">
-        <v>655</v>
+        <v>643</v>
       </c>
       <c r="D19" t="s">
         <v>323</v>
@@ -14612,21 +14658,21 @@
         <v>97</v>
       </c>
       <c r="I19" t="s">
-        <v>619</v>
+        <v>607</v>
       </c>
       <c r="J19" t="s">
-        <v>658</v>
+        <v>646</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>659</v>
+        <v>647</v>
       </c>
       <c r="B20" t="s">
-        <v>654</v>
+        <v>642</v>
       </c>
       <c r="C20" t="s">
-        <v>655</v>
+        <v>643</v>
       </c>
       <c r="D20" t="s">
         <v>323</v>
@@ -14644,21 +14690,21 @@
         <v>97</v>
       </c>
       <c r="I20" t="s">
-        <v>619</v>
+        <v>607</v>
       </c>
       <c r="J20" t="s">
-        <v>660</v>
+        <v>648</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>661</v>
+        <v>649</v>
       </c>
       <c r="B21" t="s">
-        <v>654</v>
+        <v>642</v>
       </c>
       <c r="C21" t="s">
-        <v>655</v>
+        <v>643</v>
       </c>
       <c r="D21" t="s">
         <v>323</v>
@@ -14676,21 +14722,21 @@
         <v>97</v>
       </c>
       <c r="I21" t="s">
-        <v>619</v>
+        <v>607</v>
       </c>
       <c r="J21" t="s">
-        <v>660</v>
+        <v>648</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>662</v>
+        <v>650</v>
       </c>
       <c r="B22" t="s">
-        <v>663</v>
+        <v>651</v>
       </c>
       <c r="C22" t="s">
-        <v>664</v>
+        <v>652</v>
       </c>
       <c r="D22" t="s">
         <v>323</v>
@@ -14708,21 +14754,21 @@
         <v>97</v>
       </c>
       <c r="I22" t="s">
-        <v>619</v>
+        <v>607</v>
       </c>
       <c r="J22" t="s">
-        <v>665</v>
+        <v>653</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>666</v>
+        <v>654</v>
       </c>
       <c r="B23" t="s">
-        <v>663</v>
+        <v>651</v>
       </c>
       <c r="C23" t="s">
-        <v>664</v>
+        <v>652</v>
       </c>
       <c r="D23" t="s">
         <v>323</v>
@@ -14740,21 +14786,21 @@
         <v>97</v>
       </c>
       <c r="I23" t="s">
-        <v>619</v>
+        <v>607</v>
       </c>
       <c r="J23" t="s">
-        <v>667</v>
+        <v>655</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>668</v>
+        <v>656</v>
       </c>
       <c r="B24" t="s">
-        <v>663</v>
+        <v>651</v>
       </c>
       <c r="C24" t="s">
-        <v>664</v>
+        <v>652</v>
       </c>
       <c r="D24" t="s">
         <v>323</v>
@@ -14772,21 +14818,21 @@
         <v>97</v>
       </c>
       <c r="I24" t="s">
-        <v>619</v>
+        <v>607</v>
       </c>
       <c r="J24" t="s">
-        <v>669</v>
+        <v>657</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>670</v>
+        <v>658</v>
       </c>
       <c r="B25" t="s">
-        <v>663</v>
+        <v>651</v>
       </c>
       <c r="C25" t="s">
-        <v>664</v>
+        <v>652</v>
       </c>
       <c r="D25" t="s">
         <v>323</v>
@@ -14804,10 +14850,10 @@
         <v>97</v>
       </c>
       <c r="I25" t="s">
-        <v>619</v>
+        <v>607</v>
       </c>
       <c r="J25" t="s">
-        <v>669</v>
+        <v>657</v>
       </c>
     </row>
   </sheetData>
@@ -14815,7 +14861,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.86328125" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
@@ -14825,28 +14871,28 @@
   <sheetData>
     <row r="1" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
-        <v>671</v>
+        <v>659</v>
       </c>
       <c r="B1" t="s">
-        <v>672</v>
+        <v>660</v>
       </c>
       <c r="C1" t="s">
-        <v>673</v>
+        <v>661</v>
       </c>
       <c r="D1" t="s">
-        <v>674</v>
+        <v>662</v>
       </c>
       <c r="E1" t="s">
-        <v>675</v>
+        <v>663</v>
       </c>
       <c r="F1" t="s">
-        <v>676</v>
+        <v>664</v>
       </c>
       <c r="G1" t="s">
-        <v>677</v>
+        <v>665</v>
       </c>
       <c r="H1" t="s">
-        <v>678</v>
+        <v>666</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.45">
@@ -14854,25 +14900,25 @@
         <v>115</v>
       </c>
       <c r="B2" t="s">
-        <v>679</v>
+        <v>667</v>
       </c>
       <c r="C2" t="s">
-        <v>680</v>
+        <v>668</v>
       </c>
       <c r="D2" t="s">
-        <v>681</v>
+        <v>669</v>
       </c>
       <c r="E2" t="s">
-        <v>682</v>
+        <v>670</v>
       </c>
       <c r="F2" t="s">
         <v>116</v>
       </c>
       <c r="G2" t="s">
-        <v>683</v>
+        <v>671</v>
       </c>
       <c r="H2" t="s">
-        <v>683</v>
+        <v>671</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.45">
@@ -14880,25 +14926,25 @@
         <v>184</v>
       </c>
       <c r="B3" t="s">
-        <v>684</v>
+        <v>672</v>
       </c>
       <c r="C3" t="s">
-        <v>680</v>
+        <v>668</v>
       </c>
       <c r="D3" t="s">
         <v>182</v>
       </c>
       <c r="E3" t="s">
-        <v>685</v>
+        <v>673</v>
       </c>
       <c r="F3" t="s">
         <v>185</v>
       </c>
       <c r="G3" t="s">
-        <v>683</v>
+        <v>671</v>
       </c>
       <c r="H3" t="s">
-        <v>683</v>
+        <v>671</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.45">
@@ -14906,25 +14952,25 @@
         <v>126</v>
       </c>
       <c r="B4" t="s">
-        <v>686</v>
+        <v>674</v>
       </c>
       <c r="C4" t="s">
-        <v>687</v>
+        <v>675</v>
       </c>
       <c r="D4" t="s">
-        <v>688</v>
+        <v>676</v>
       </c>
       <c r="E4" t="s">
-        <v>689</v>
+        <v>677</v>
       </c>
       <c r="F4" t="s">
         <v>127</v>
       </c>
       <c r="G4" t="s">
-        <v>683</v>
+        <v>671</v>
       </c>
       <c r="H4" t="s">
-        <v>690</v>
+        <v>678</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.45">
@@ -14932,381 +14978,25 @@
         <v>64</v>
       </c>
       <c r="B5" t="s">
-        <v>691</v>
+        <v>679</v>
       </c>
       <c r="C5" t="s">
-        <v>692</v>
+        <v>680</v>
       </c>
       <c r="D5" t="s">
-        <v>693</v>
+        <v>681</v>
       </c>
       <c r="E5" t="s">
-        <v>694</v>
+        <v>682</v>
       </c>
       <c r="F5" t="s">
         <v>65</v>
       </c>
       <c r="G5" t="s">
-        <v>683</v>
+        <v>671</v>
       </c>
       <c r="H5" t="s">
-        <v>690</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:C11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.86328125" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
-  <sheetData>
-    <row r="1" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" t="s">
-        <v>695</v>
-      </c>
-      <c r="B1" t="s">
-        <v>696</v>
-      </c>
-      <c r="C1" t="s">
-        <v>697</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
-        <v>698</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>699</v>
-      </c>
-      <c r="B3" t="s">
-        <v>700</v>
-      </c>
-      <c r="C3" t="s">
-        <v>701</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>702</v>
-      </c>
-      <c r="B4" t="s">
-        <v>700</v>
-      </c>
-      <c r="C4" t="s">
-        <v>701</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>703</v>
-      </c>
-      <c r="B5" t="s">
-        <v>700</v>
-      </c>
-      <c r="C5" t="s">
-        <v>701</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>704</v>
-      </c>
-      <c r="B6" t="s">
-        <v>700</v>
-      </c>
-      <c r="C6" t="s">
-        <v>701</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>705</v>
-      </c>
-      <c r="B7" t="s">
-        <v>700</v>
-      </c>
-      <c r="C7" t="s">
-        <v>701</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>706</v>
-      </c>
-      <c r="B8" t="s">
-        <v>700</v>
-      </c>
-      <c r="C8" t="s">
-        <v>701</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>707</v>
-      </c>
-      <c r="B9" t="s">
-        <v>700</v>
-      </c>
-      <c r="C9" t="s">
-        <v>701</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>708</v>
-      </c>
-      <c r="B10" t="s">
-        <v>709</v>
-      </c>
-      <c r="C10" t="s">
-        <v>701</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A11" t="s">
-        <v>710</v>
-      </c>
-      <c r="B11" t="s">
-        <v>711</v>
-      </c>
-      <c r="C11" t="s">
-        <v>701</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:E13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.86328125" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
-  <sheetData>
-    <row r="1" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" t="s">
-        <v>712</v>
-      </c>
-      <c r="B1" t="s">
-        <v>713</v>
-      </c>
-      <c r="C1" t="s">
-        <v>714</v>
-      </c>
-      <c r="D1" t="s">
-        <v>715</v>
-      </c>
-      <c r="E1" t="s">
-        <v>716</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
-        <v>717</v>
-      </c>
-      <c r="B2" t="s">
-        <v>718</v>
-      </c>
-      <c r="C2" t="s">
-        <v>719</v>
-      </c>
-      <c r="D2" t="s">
-        <v>720</v>
-      </c>
-      <c r="E2" t="s">
-        <v>721</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>717</v>
-      </c>
-      <c r="B3" t="s">
-        <v>722</v>
-      </c>
-      <c r="C3" t="s">
-        <v>723</v>
-      </c>
-      <c r="D3" t="s">
-        <v>724</v>
-      </c>
-      <c r="E3" t="s">
-        <v>725</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
-        <v>717</v>
-      </c>
-      <c r="B4" t="s">
-        <v>722</v>
-      </c>
-      <c r="C4" t="s">
-        <v>726</v>
-      </c>
-      <c r="D4" t="s">
-        <v>727</v>
-      </c>
-      <c r="E4" t="s">
-        <v>728</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A5" t="s">
-        <v>717</v>
-      </c>
-      <c r="B5" t="s">
-        <v>729</v>
-      </c>
-      <c r="C5" t="s">
-        <v>730</v>
-      </c>
-      <c r="D5" t="s">
-        <v>731</v>
-      </c>
-      <c r="E5" t="s">
-        <v>732</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>733</v>
-      </c>
-      <c r="B6" t="s">
-        <v>734</v>
-      </c>
-      <c r="C6" t="s">
-        <v>735</v>
-      </c>
-      <c r="D6" t="s">
-        <v>736</v>
-      </c>
-      <c r="E6" t="s">
-        <v>737</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>733</v>
-      </c>
-      <c r="B7" t="s">
-        <v>734</v>
-      </c>
-      <c r="C7" t="s">
-        <v>738</v>
-      </c>
-      <c r="D7" t="s">
-        <v>739</v>
-      </c>
-      <c r="E7" t="s">
-        <v>740</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A8" t="s">
-        <v>733</v>
-      </c>
-      <c r="B8" t="s">
-        <v>741</v>
-      </c>
-      <c r="C8" t="s">
-        <v>742</v>
-      </c>
-      <c r="D8" t="s">
-        <v>743</v>
-      </c>
-      <c r="E8" t="s">
-        <v>744</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A9" t="s">
-        <v>733</v>
-      </c>
-      <c r="B9" t="s">
-        <v>741</v>
-      </c>
-      <c r="C9" t="s">
-        <v>745</v>
-      </c>
-      <c r="D9" t="s">
-        <v>746</v>
-      </c>
-      <c r="E9" t="s">
-        <v>744</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A10" t="s">
-        <v>747</v>
-      </c>
-      <c r="B10" t="s">
-        <v>748</v>
-      </c>
-      <c r="C10" t="s">
-        <v>749</v>
-      </c>
-      <c r="D10" t="s">
-        <v>750</v>
-      </c>
-      <c r="E10" t="s">
-        <v>751</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A11" t="s">
-        <v>747</v>
-      </c>
-      <c r="B11" t="s">
-        <v>752</v>
-      </c>
-      <c r="C11" t="s">
-        <v>753</v>
-      </c>
-      <c r="D11" t="s">
-        <v>754</v>
-      </c>
-      <c r="E11" t="s">
-        <v>755</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A12" t="s">
-        <v>747</v>
-      </c>
-      <c r="B12" t="s">
-        <v>752</v>
-      </c>
-      <c r="C12" t="s">
-        <v>127</v>
-      </c>
-      <c r="D12" t="s">
-        <v>754</v>
-      </c>
-      <c r="E12" t="s">
-        <v>756</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A13" t="s">
-        <v>747</v>
-      </c>
-      <c r="B13" t="s">
-        <v>752</v>
-      </c>
-      <c r="C13" t="s">
-        <v>757</v>
-      </c>
-      <c r="D13" t="s">
-        <v>754</v>
-      </c>
-      <c r="E13" t="s">
-        <v>758</v>
+        <v>678</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Agrega emails transaccionales (confirmación + envío) y panel /admin
Implementa los flujos de correo vía Resend/react-email disparados desde
un webhook de Supabase sobre orders, y un panel /admin con auth por
whitelist para que Anahí/JCC capturen guía de envío sin tocar la base
de datos a mano.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Catalogo_Master_Lhopital-moto.xlsx
+++ b/Catalogo_Master_Lhopital-moto.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\lhopital-moto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0944B61-EC45-4B31-AB02-D3842D4FB6FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{484C1175-1B25-4768-BBC6-F8920702FE78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LÉEME" sheetId="1" r:id="rId1"/>
@@ -2755,7 +2755,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2780,6 +2780,7 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Moneda" xfId="1" builtinId="4"/>
@@ -4014,7 +4015,10 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.86328125" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="15.33203125" customWidth="1"/>
-    <col min="4" max="4" width="26.33203125" customWidth="1"/>
+    <col min="3" max="4" width="15.796875" customWidth="1"/>
+    <col min="5" max="5" width="5.9296875" customWidth="1"/>
+    <col min="6" max="6" width="10.86328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.1328125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="33.1328125" customWidth="1"/>
     <col min="15" max="15" width="26.9296875" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="30" customWidth="1"/>
@@ -4089,7 +4093,7 @@
       <c r="E2" t="s">
         <v>69</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="14">
         <v>12600</v>
       </c>
       <c r="G2">
@@ -4130,7 +4134,7 @@
       <c r="E3" t="s">
         <v>77</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="14">
         <v>12600</v>
       </c>
       <c r="G3">
@@ -4171,7 +4175,7 @@
       <c r="E4" t="s">
         <v>79</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="14">
         <v>12600</v>
       </c>
       <c r="G4">
@@ -4212,7 +4216,7 @@
       <c r="E5" t="s">
         <v>81</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="14">
         <v>12600</v>
       </c>
       <c r="G5">
@@ -4253,7 +4257,7 @@
       <c r="E6" t="s">
         <v>83</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="14">
         <v>12600</v>
       </c>
       <c r="G6">
@@ -4294,7 +4298,7 @@
       <c r="E7" t="s">
         <v>85</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="14">
         <v>12600</v>
       </c>
       <c r="G7">
@@ -4335,7 +4339,7 @@
       <c r="E8" t="s">
         <v>69</v>
       </c>
-      <c r="F8">
+      <c r="F8" s="14">
         <v>12600</v>
       </c>
       <c r="G8">
@@ -4379,7 +4383,7 @@
       <c r="E9" t="s">
         <v>77</v>
       </c>
-      <c r="F9">
+      <c r="F9" s="14">
         <v>12600</v>
       </c>
       <c r="G9">
@@ -4423,7 +4427,7 @@
       <c r="E10" t="s">
         <v>79</v>
       </c>
-      <c r="F10">
+      <c r="F10" s="14">
         <v>12600</v>
       </c>
       <c r="G10">
@@ -4467,7 +4471,7 @@
       <c r="E11" t="s">
         <v>81</v>
       </c>
-      <c r="F11">
+      <c r="F11" s="14">
         <v>12600</v>
       </c>
       <c r="G11">
@@ -4511,7 +4515,7 @@
       <c r="E12" t="s">
         <v>83</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="14">
         <v>12600</v>
       </c>
       <c r="G12">
@@ -4555,7 +4559,7 @@
       <c r="E13" t="s">
         <v>85</v>
       </c>
-      <c r="F13">
+      <c r="F13" s="14">
         <v>12600</v>
       </c>
       <c r="G13">
@@ -4599,7 +4603,7 @@
       <c r="E14" t="s">
         <v>69</v>
       </c>
-      <c r="F14">
+      <c r="F14" s="14">
         <v>14000</v>
       </c>
       <c r="G14">
@@ -4640,7 +4644,7 @@
       <c r="E15" t="s">
         <v>77</v>
       </c>
-      <c r="F15">
+      <c r="F15" s="14">
         <v>14000</v>
       </c>
       <c r="G15">
@@ -4681,7 +4685,7 @@
       <c r="E16" t="s">
         <v>79</v>
       </c>
-      <c r="F16">
+      <c r="F16" s="14">
         <v>14000</v>
       </c>
       <c r="G16">
@@ -4722,7 +4726,7 @@
       <c r="E17" t="s">
         <v>81</v>
       </c>
-      <c r="F17">
+      <c r="F17" s="14">
         <v>14000</v>
       </c>
       <c r="G17">
@@ -4763,7 +4767,7 @@
       <c r="E18" t="s">
         <v>83</v>
       </c>
-      <c r="F18">
+      <c r="F18" s="14">
         <v>14000</v>
       </c>
       <c r="G18">
@@ -4804,7 +4808,7 @@
       <c r="E19" t="s">
         <v>85</v>
       </c>
-      <c r="F19">
+      <c r="F19" s="14">
         <v>14000</v>
       </c>
       <c r="G19">
@@ -4845,7 +4849,7 @@
       <c r="E20" t="s">
         <v>69</v>
       </c>
-      <c r="F20">
+      <c r="F20" s="14">
         <v>14000</v>
       </c>
       <c r="G20">
@@ -4889,7 +4893,7 @@
       <c r="E21" t="s">
         <v>77</v>
       </c>
-      <c r="F21">
+      <c r="F21" s="14">
         <v>14000</v>
       </c>
       <c r="G21">
@@ -4933,7 +4937,7 @@
       <c r="E22" t="s">
         <v>79</v>
       </c>
-      <c r="F22">
+      <c r="F22" s="14">
         <v>14000</v>
       </c>
       <c r="G22">
@@ -4977,7 +4981,7 @@
       <c r="E23" t="s">
         <v>81</v>
       </c>
-      <c r="F23">
+      <c r="F23" s="14">
         <v>14000</v>
       </c>
       <c r="G23">
@@ -5021,7 +5025,7 @@
       <c r="E24" t="s">
         <v>83</v>
       </c>
-      <c r="F24">
+      <c r="F24" s="14">
         <v>14000</v>
       </c>
       <c r="G24">
@@ -5065,7 +5069,7 @@
       <c r="E25" t="s">
         <v>85</v>
       </c>
-      <c r="F25">
+      <c r="F25" s="14">
         <v>14000</v>
       </c>
       <c r="G25">
@@ -5109,7 +5113,7 @@
       <c r="E26" t="s">
         <v>69</v>
       </c>
-      <c r="F26">
+      <c r="F26" s="14">
         <v>14000</v>
       </c>
       <c r="G26">
@@ -5147,7 +5151,7 @@
       <c r="E27" t="s">
         <v>77</v>
       </c>
-      <c r="F27">
+      <c r="F27" s="14">
         <v>14000</v>
       </c>
       <c r="G27">
@@ -5185,7 +5189,7 @@
       <c r="E28" t="s">
         <v>79</v>
       </c>
-      <c r="F28">
+      <c r="F28" s="14">
         <v>14000</v>
       </c>
       <c r="G28">
@@ -5223,7 +5227,7 @@
       <c r="E29" t="s">
         <v>81</v>
       </c>
-      <c r="F29">
+      <c r="F29" s="14">
         <v>14000</v>
       </c>
       <c r="G29">
@@ -5261,7 +5265,7 @@
       <c r="E30" t="s">
         <v>83</v>
       </c>
-      <c r="F30">
+      <c r="F30" s="14">
         <v>14000</v>
       </c>
       <c r="G30">
@@ -5299,7 +5303,7 @@
       <c r="E31" t="s">
         <v>85</v>
       </c>
-      <c r="F31">
+      <c r="F31" s="14">
         <v>14000</v>
       </c>
       <c r="G31">
@@ -5337,7 +5341,7 @@
       <c r="E32" t="s">
         <v>69</v>
       </c>
-      <c r="F32">
+      <c r="F32" s="14">
         <v>16000</v>
       </c>
       <c r="G32">
@@ -5378,7 +5382,7 @@
       <c r="E33" t="s">
         <v>77</v>
       </c>
-      <c r="F33">
+      <c r="F33" s="14">
         <v>16000</v>
       </c>
       <c r="G33">
@@ -5419,7 +5423,7 @@
       <c r="E34" t="s">
         <v>79</v>
       </c>
-      <c r="F34">
+      <c r="F34" s="14">
         <v>16000</v>
       </c>
       <c r="G34">
@@ -5460,7 +5464,7 @@
       <c r="E35" t="s">
         <v>81</v>
       </c>
-      <c r="F35">
+      <c r="F35" s="14">
         <v>16000</v>
       </c>
       <c r="G35">
@@ -5501,7 +5505,7 @@
       <c r="E36" t="s">
         <v>83</v>
       </c>
-      <c r="F36">
+      <c r="F36" s="14">
         <v>16000</v>
       </c>
       <c r="G36">
@@ -5542,7 +5546,7 @@
       <c r="E37" t="s">
         <v>85</v>
       </c>
-      <c r="F37">
+      <c r="F37" s="14">
         <v>16000</v>
       </c>
       <c r="G37">
@@ -5583,7 +5587,7 @@
       <c r="E38" t="s">
         <v>69</v>
       </c>
-      <c r="F38">
+      <c r="F38" s="14">
         <v>16000</v>
       </c>
       <c r="G38">
@@ -5621,7 +5625,7 @@
       <c r="E39" t="s">
         <v>77</v>
       </c>
-      <c r="F39">
+      <c r="F39" s="14">
         <v>16000</v>
       </c>
       <c r="G39">
@@ -5659,7 +5663,7 @@
       <c r="E40" t="s">
         <v>79</v>
       </c>
-      <c r="F40">
+      <c r="F40" s="14">
         <v>16000</v>
       </c>
       <c r="G40">
@@ -5697,7 +5701,7 @@
       <c r="E41" t="s">
         <v>81</v>
       </c>
-      <c r="F41">
+      <c r="F41" s="14">
         <v>16000</v>
       </c>
       <c r="G41">
@@ -5735,7 +5739,7 @@
       <c r="E42" t="s">
         <v>83</v>
       </c>
-      <c r="F42">
+      <c r="F42" s="14">
         <v>16000</v>
       </c>
       <c r="G42">
@@ -5773,7 +5777,7 @@
       <c r="E43" t="s">
         <v>85</v>
       </c>
-      <c r="F43">
+      <c r="F43" s="14">
         <v>16000</v>
       </c>
       <c r="G43">
@@ -5811,7 +5815,7 @@
       <c r="E44" t="s">
         <v>69</v>
       </c>
-      <c r="F44">
+      <c r="F44" s="14">
         <v>17500</v>
       </c>
       <c r="G44">
@@ -5849,7 +5853,7 @@
       <c r="E45" t="s">
         <v>77</v>
       </c>
-      <c r="F45">
+      <c r="F45" s="14">
         <v>17500</v>
       </c>
       <c r="G45">
@@ -5887,7 +5891,7 @@
       <c r="E46" t="s">
         <v>79</v>
       </c>
-      <c r="F46">
+      <c r="F46" s="14">
         <v>17500</v>
       </c>
       <c r="G46">
@@ -5925,7 +5929,7 @@
       <c r="E47" t="s">
         <v>81</v>
       </c>
-      <c r="F47">
+      <c r="F47" s="14">
         <v>17500</v>
       </c>
       <c r="G47">
@@ -5963,7 +5967,7 @@
       <c r="E48" t="s">
         <v>83</v>
       </c>
-      <c r="F48">
+      <c r="F48" s="14">
         <v>17500</v>
       </c>
       <c r="G48">
@@ -6001,7 +6005,7 @@
       <c r="E49" t="s">
         <v>85</v>
       </c>
-      <c r="F49">
+      <c r="F49" s="14">
         <v>17500</v>
       </c>
       <c r="G49">
@@ -6039,7 +6043,7 @@
       <c r="E50" t="s">
         <v>69</v>
       </c>
-      <c r="F50">
+      <c r="F50" s="14">
         <v>17000</v>
       </c>
       <c r="G50">
@@ -6077,7 +6081,7 @@
       <c r="E51" t="s">
         <v>77</v>
       </c>
-      <c r="F51">
+      <c r="F51" s="14">
         <v>17000</v>
       </c>
       <c r="G51">
@@ -6115,7 +6119,7 @@
       <c r="E52" t="s">
         <v>79</v>
       </c>
-      <c r="F52">
+      <c r="F52" s="14">
         <v>17000</v>
       </c>
       <c r="G52">
@@ -6153,7 +6157,7 @@
       <c r="E53" t="s">
         <v>81</v>
       </c>
-      <c r="F53">
+      <c r="F53" s="14">
         <v>17000</v>
       </c>
       <c r="G53">
@@ -6191,7 +6195,7 @@
       <c r="E54" t="s">
         <v>83</v>
       </c>
-      <c r="F54">
+      <c r="F54" s="14">
         <v>17000</v>
       </c>
       <c r="G54">
@@ -6229,7 +6233,7 @@
       <c r="E55" t="s">
         <v>85</v>
       </c>
-      <c r="F55">
+      <c r="F55" s="14">
         <v>17000</v>
       </c>
       <c r="G55">
@@ -6267,7 +6271,7 @@
       <c r="E56" t="s">
         <v>69</v>
       </c>
-      <c r="F56">
+      <c r="F56" s="14">
         <v>17000</v>
       </c>
       <c r="G56">
@@ -6308,7 +6312,7 @@
       <c r="E57" t="s">
         <v>77</v>
       </c>
-      <c r="F57">
+      <c r="F57" s="14">
         <v>17000</v>
       </c>
       <c r="G57">
@@ -6349,7 +6353,7 @@
       <c r="E58" t="s">
         <v>79</v>
       </c>
-      <c r="F58">
+      <c r="F58" s="14">
         <v>17000</v>
       </c>
       <c r="G58">
@@ -6390,7 +6394,7 @@
       <c r="E59" t="s">
         <v>81</v>
       </c>
-      <c r="F59">
+      <c r="F59" s="14">
         <v>17000</v>
       </c>
       <c r="G59">
@@ -6431,7 +6435,7 @@
       <c r="E60" t="s">
         <v>83</v>
       </c>
-      <c r="F60">
+      <c r="F60" s="14">
         <v>17000</v>
       </c>
       <c r="G60">
@@ -6472,7 +6476,7 @@
       <c r="E61" t="s">
         <v>85</v>
       </c>
-      <c r="F61">
+      <c r="F61" s="14">
         <v>17000</v>
       </c>
       <c r="G61">
@@ -6513,7 +6517,7 @@
       <c r="E62" t="s">
         <v>69</v>
       </c>
-      <c r="F62">
+      <c r="F62" s="14">
         <v>18700</v>
       </c>
       <c r="G62">
@@ -6551,7 +6555,7 @@
       <c r="E63" t="s">
         <v>77</v>
       </c>
-      <c r="F63">
+      <c r="F63" s="14">
         <v>18700</v>
       </c>
       <c r="G63">
@@ -6589,7 +6593,7 @@
       <c r="E64" t="s">
         <v>79</v>
       </c>
-      <c r="F64">
+      <c r="F64" s="14">
         <v>18700</v>
       </c>
       <c r="G64">
@@ -6627,7 +6631,7 @@
       <c r="E65" t="s">
         <v>81</v>
       </c>
-      <c r="F65">
+      <c r="F65" s="14">
         <v>18700</v>
       </c>
       <c r="G65">
@@ -6665,7 +6669,7 @@
       <c r="E66" t="s">
         <v>83</v>
       </c>
-      <c r="F66">
+      <c r="F66" s="14">
         <v>18700</v>
       </c>
       <c r="G66">
@@ -6703,7 +6707,7 @@
       <c r="E67" t="s">
         <v>85</v>
       </c>
-      <c r="F67">
+      <c r="F67" s="14">
         <v>18700</v>
       </c>
       <c r="G67">
@@ -6741,8 +6745,8 @@
       <c r="E68" t="s">
         <v>69</v>
       </c>
-      <c r="F68">
-        <v>25500</v>
+      <c r="F68" s="14">
+        <v>33000</v>
       </c>
       <c r="G68">
         <v>0</v>
@@ -6779,8 +6783,8 @@
       <c r="E69" t="s">
         <v>77</v>
       </c>
-      <c r="F69">
-        <v>25500</v>
+      <c r="F69" s="14">
+        <v>33000</v>
       </c>
       <c r="G69">
         <v>0</v>
@@ -6817,8 +6821,8 @@
       <c r="E70" t="s">
         <v>79</v>
       </c>
-      <c r="F70">
-        <v>25500</v>
+      <c r="F70" s="14">
+        <v>33000</v>
       </c>
       <c r="G70">
         <v>0</v>
@@ -6855,8 +6859,8 @@
       <c r="E71" t="s">
         <v>81</v>
       </c>
-      <c r="F71">
-        <v>25500</v>
+      <c r="F71" s="14">
+        <v>33000</v>
       </c>
       <c r="G71">
         <v>0</v>
@@ -6893,8 +6897,8 @@
       <c r="E72" t="s">
         <v>83</v>
       </c>
-      <c r="F72">
-        <v>25500</v>
+      <c r="F72" s="14">
+        <v>33000</v>
       </c>
       <c r="G72">
         <v>0</v>
@@ -6931,8 +6935,8 @@
       <c r="E73" t="s">
         <v>85</v>
       </c>
-      <c r="F73">
-        <v>25500</v>
+      <c r="F73" s="14">
+        <v>33000</v>
       </c>
       <c r="G73">
         <v>0</v>
@@ -6969,8 +6973,8 @@
       <c r="E74" t="s">
         <v>69</v>
       </c>
-      <c r="F74">
-        <v>25500</v>
+      <c r="F74" s="14">
+        <v>33000</v>
       </c>
       <c r="G74">
         <v>0</v>
@@ -7010,8 +7014,8 @@
       <c r="E75" t="s">
         <v>77</v>
       </c>
-      <c r="F75">
-        <v>25500</v>
+      <c r="F75" s="14">
+        <v>33000</v>
       </c>
       <c r="G75">
         <v>0</v>
@@ -7051,8 +7055,8 @@
       <c r="E76" t="s">
         <v>79</v>
       </c>
-      <c r="F76">
-        <v>25500</v>
+      <c r="F76" s="14">
+        <v>33000</v>
       </c>
       <c r="G76">
         <v>0</v>
@@ -7092,8 +7096,8 @@
       <c r="E77" t="s">
         <v>81</v>
       </c>
-      <c r="F77">
-        <v>25500</v>
+      <c r="F77" s="14">
+        <v>33000</v>
       </c>
       <c r="G77">
         <v>0</v>
@@ -7133,8 +7137,8 @@
       <c r="E78" t="s">
         <v>83</v>
       </c>
-      <c r="F78">
-        <v>25500</v>
+      <c r="F78" s="14">
+        <v>33000</v>
       </c>
       <c r="G78">
         <v>0</v>
@@ -7174,8 +7178,8 @@
       <c r="E79" t="s">
         <v>85</v>
       </c>
-      <c r="F79">
-        <v>25500</v>
+      <c r="F79" s="14">
+        <v>33000</v>
       </c>
       <c r="G79">
         <v>0</v>
@@ -7215,8 +7219,8 @@
       <c r="E80" t="s">
         <v>69</v>
       </c>
-      <c r="F80">
-        <v>28350</v>
+      <c r="F80" s="14">
+        <v>35000</v>
       </c>
       <c r="G80">
         <v>0</v>
@@ -7253,8 +7257,8 @@
       <c r="E81" t="s">
         <v>77</v>
       </c>
-      <c r="F81">
-        <v>28350</v>
+      <c r="F81" s="14">
+        <v>35000</v>
       </c>
       <c r="G81">
         <v>0</v>
@@ -7291,8 +7295,8 @@
       <c r="E82" t="s">
         <v>79</v>
       </c>
-      <c r="F82">
-        <v>28350</v>
+      <c r="F82" s="14">
+        <v>35000</v>
       </c>
       <c r="G82">
         <v>0</v>
@@ -7329,8 +7333,8 @@
       <c r="E83" t="s">
         <v>81</v>
       </c>
-      <c r="F83">
-        <v>28350</v>
+      <c r="F83" s="14">
+        <v>35000</v>
       </c>
       <c r="G83">
         <v>0</v>
@@ -7367,8 +7371,8 @@
       <c r="E84" t="s">
         <v>83</v>
       </c>
-      <c r="F84">
-        <v>28350</v>
+      <c r="F84" s="14">
+        <v>35000</v>
       </c>
       <c r="G84">
         <v>0</v>
@@ -7405,8 +7409,8 @@
       <c r="E85" t="s">
         <v>85</v>
       </c>
-      <c r="F85">
-        <v>28350</v>
+      <c r="F85" s="14">
+        <v>35000</v>
       </c>
       <c r="G85">
         <v>0</v>
@@ -7443,7 +7447,7 @@
       <c r="E86" t="s">
         <v>69</v>
       </c>
-      <c r="F86">
+      <c r="F86" s="14">
         <v>22900</v>
       </c>
       <c r="G86">
@@ -7484,7 +7488,7 @@
       <c r="E87" t="s">
         <v>77</v>
       </c>
-      <c r="F87">
+      <c r="F87" s="14">
         <v>22900</v>
       </c>
       <c r="G87">
@@ -7525,7 +7529,7 @@
       <c r="E88" t="s">
         <v>79</v>
       </c>
-      <c r="F88">
+      <c r="F88" s="14">
         <v>22900</v>
       </c>
       <c r="G88">
@@ -7566,7 +7570,7 @@
       <c r="E89" t="s">
         <v>81</v>
       </c>
-      <c r="F89">
+      <c r="F89" s="14">
         <v>22900</v>
       </c>
       <c r="G89">
@@ -7607,7 +7611,7 @@
       <c r="E90" t="s">
         <v>83</v>
       </c>
-      <c r="F90">
+      <c r="F90" s="14">
         <v>22900</v>
       </c>
       <c r="G90">
@@ -7648,7 +7652,7 @@
       <c r="E91" t="s">
         <v>85</v>
       </c>
-      <c r="F91">
+      <c r="F91" s="14">
         <v>22900</v>
       </c>
       <c r="G91">
@@ -7689,7 +7693,7 @@
       <c r="E92" t="s">
         <v>69</v>
       </c>
-      <c r="F92">
+      <c r="F92" s="14">
         <v>24200</v>
       </c>
       <c r="G92">
@@ -7727,7 +7731,7 @@
       <c r="E93" t="s">
         <v>77</v>
       </c>
-      <c r="F93">
+      <c r="F93" s="14">
         <v>24200</v>
       </c>
       <c r="G93">
@@ -7765,7 +7769,7 @@
       <c r="E94" t="s">
         <v>79</v>
       </c>
-      <c r="F94">
+      <c r="F94" s="14">
         <v>24200</v>
       </c>
       <c r="G94">
@@ -7803,7 +7807,7 @@
       <c r="E95" t="s">
         <v>81</v>
       </c>
-      <c r="F95">
+      <c r="F95" s="14">
         <v>24200</v>
       </c>
       <c r="G95">
@@ -7841,7 +7845,7 @@
       <c r="E96" t="s">
         <v>83</v>
       </c>
-      <c r="F96">
+      <c r="F96" s="14">
         <v>24200</v>
       </c>
       <c r="G96">
@@ -7879,7 +7883,7 @@
       <c r="E97" t="s">
         <v>85</v>
       </c>
-      <c r="F97">
+      <c r="F97" s="14">
         <v>24200</v>
       </c>
       <c r="G97">
@@ -7917,7 +7921,7 @@
       <c r="E98" t="s">
         <v>69</v>
       </c>
-      <c r="F98">
+      <c r="F98" s="14">
         <v>24200</v>
       </c>
       <c r="G98">
@@ -7955,7 +7959,7 @@
       <c r="E99" t="s">
         <v>77</v>
       </c>
-      <c r="F99">
+      <c r="F99" s="14">
         <v>24200</v>
       </c>
       <c r="G99">
@@ -7993,7 +7997,7 @@
       <c r="E100" t="s">
         <v>79</v>
       </c>
-      <c r="F100">
+      <c r="F100" s="14">
         <v>24200</v>
       </c>
       <c r="G100">
@@ -8031,7 +8035,7 @@
       <c r="E101" t="s">
         <v>81</v>
       </c>
-      <c r="F101">
+      <c r="F101" s="14">
         <v>24200</v>
       </c>
       <c r="G101">
@@ -8069,7 +8073,7 @@
       <c r="E102" t="s">
         <v>83</v>
       </c>
-      <c r="F102">
+      <c r="F102" s="14">
         <v>24200</v>
       </c>
       <c r="G102">
@@ -8107,7 +8111,7 @@
       <c r="E103" t="s">
         <v>85</v>
       </c>
-      <c r="F103">
+      <c r="F103" s="14">
         <v>24200</v>
       </c>
       <c r="G103">
@@ -8145,7 +8149,7 @@
       <c r="E104" t="s">
         <v>69</v>
       </c>
-      <c r="F104">
+      <c r="F104" s="14">
         <v>24200</v>
       </c>
       <c r="G104">
@@ -8189,7 +8193,7 @@
       <c r="E105" t="s">
         <v>77</v>
       </c>
-      <c r="F105">
+      <c r="F105" s="14">
         <v>24200</v>
       </c>
       <c r="G105">
@@ -8233,7 +8237,7 @@
       <c r="E106" t="s">
         <v>79</v>
       </c>
-      <c r="F106">
+      <c r="F106" s="14">
         <v>24200</v>
       </c>
       <c r="G106">
@@ -8277,7 +8281,7 @@
       <c r="E107" t="s">
         <v>81</v>
       </c>
-      <c r="F107">
+      <c r="F107" s="14">
         <v>24200</v>
       </c>
       <c r="G107">
@@ -8321,7 +8325,7 @@
       <c r="E108" t="s">
         <v>83</v>
       </c>
-      <c r="F108">
+      <c r="F108" s="14">
         <v>24200</v>
       </c>
       <c r="G108">
@@ -8365,7 +8369,7 @@
       <c r="E109" t="s">
         <v>85</v>
       </c>
-      <c r="F109">
+      <c r="F109" s="14">
         <v>24200</v>
       </c>
       <c r="G109">
@@ -8409,7 +8413,7 @@
       <c r="E110" t="s">
         <v>69</v>
       </c>
-      <c r="F110">
+      <c r="F110" s="14">
         <v>24200</v>
       </c>
       <c r="G110">
@@ -8450,7 +8454,7 @@
       <c r="E111" t="s">
         <v>77</v>
       </c>
-      <c r="F111">
+      <c r="F111" s="14">
         <v>24200</v>
       </c>
       <c r="G111">
@@ -8491,7 +8495,7 @@
       <c r="E112" t="s">
         <v>79</v>
       </c>
-      <c r="F112">
+      <c r="F112" s="14">
         <v>24200</v>
       </c>
       <c r="G112">
@@ -8532,7 +8536,7 @@
       <c r="E113" t="s">
         <v>81</v>
       </c>
-      <c r="F113">
+      <c r="F113" s="14">
         <v>24200</v>
       </c>
       <c r="G113">
@@ -8573,7 +8577,7 @@
       <c r="E114" t="s">
         <v>83</v>
       </c>
-      <c r="F114">
+      <c r="F114" s="14">
         <v>24200</v>
       </c>
       <c r="G114">
@@ -8614,7 +8618,7 @@
       <c r="E115" t="s">
         <v>85</v>
       </c>
-      <c r="F115">
+      <c r="F115" s="14">
         <v>24200</v>
       </c>
       <c r="G115">
@@ -8655,7 +8659,7 @@
       <c r="E116" t="s">
         <v>69</v>
       </c>
-      <c r="F116">
+      <c r="F116" s="14">
         <v>26900</v>
       </c>
       <c r="G116">
@@ -8693,7 +8697,7 @@
       <c r="E117" t="s">
         <v>77</v>
       </c>
-      <c r="F117">
+      <c r="F117" s="14">
         <v>26900</v>
       </c>
       <c r="G117">
@@ -8731,7 +8735,7 @@
       <c r="E118" t="s">
         <v>79</v>
       </c>
-      <c r="F118">
+      <c r="F118" s="14">
         <v>26900</v>
       </c>
       <c r="G118">
@@ -8769,7 +8773,7 @@
       <c r="E119" t="s">
         <v>81</v>
       </c>
-      <c r="F119">
+      <c r="F119" s="14">
         <v>26900</v>
       </c>
       <c r="G119">
@@ -8807,7 +8811,7 @@
       <c r="E120" t="s">
         <v>83</v>
       </c>
-      <c r="F120">
+      <c r="F120" s="14">
         <v>26900</v>
       </c>
       <c r="G120">
@@ -8845,7 +8849,7 @@
       <c r="E121" t="s">
         <v>85</v>
       </c>
-      <c r="F121">
+      <c r="F121" s="14">
         <v>26900</v>
       </c>
       <c r="G121">
@@ -8883,7 +8887,7 @@
       <c r="E122" t="s">
         <v>69</v>
       </c>
-      <c r="F122">
+      <c r="F122" s="14">
         <v>26900</v>
       </c>
       <c r="G122">
@@ -8924,7 +8928,7 @@
       <c r="E123" t="s">
         <v>77</v>
       </c>
-      <c r="F123">
+      <c r="F123" s="14">
         <v>26900</v>
       </c>
       <c r="G123">
@@ -8965,7 +8969,7 @@
       <c r="E124" t="s">
         <v>79</v>
       </c>
-      <c r="F124">
+      <c r="F124" s="14">
         <v>26900</v>
       </c>
       <c r="G124">
@@ -9006,7 +9010,7 @@
       <c r="E125" t="s">
         <v>81</v>
       </c>
-      <c r="F125">
+      <c r="F125" s="14">
         <v>26900</v>
       </c>
       <c r="G125">
@@ -9047,7 +9051,7 @@
       <c r="E126" t="s">
         <v>83</v>
       </c>
-      <c r="F126">
+      <c r="F126" s="14">
         <v>26900</v>
       </c>
       <c r="G126">
@@ -9088,7 +9092,7 @@
       <c r="E127" t="s">
         <v>85</v>
       </c>
-      <c r="F127">
+      <c r="F127" s="14">
         <v>26900</v>
       </c>
       <c r="G127">
@@ -9129,7 +9133,7 @@
       <c r="E128" t="s">
         <v>69</v>
       </c>
-      <c r="F128">
+      <c r="F128" s="14">
         <v>26900</v>
       </c>
       <c r="G128">
@@ -9170,7 +9174,7 @@
       <c r="E129" t="s">
         <v>77</v>
       </c>
-      <c r="F129">
+      <c r="F129" s="14">
         <v>26900</v>
       </c>
       <c r="G129">
@@ -9211,7 +9215,7 @@
       <c r="E130" t="s">
         <v>79</v>
       </c>
-      <c r="F130">
+      <c r="F130" s="14">
         <v>26900</v>
       </c>
       <c r="G130">
@@ -9252,7 +9256,7 @@
       <c r="E131" t="s">
         <v>81</v>
       </c>
-      <c r="F131">
+      <c r="F131" s="14">
         <v>26900</v>
       </c>
       <c r="G131">
@@ -9293,7 +9297,7 @@
       <c r="E132" t="s">
         <v>83</v>
       </c>
-      <c r="F132">
+      <c r="F132" s="14">
         <v>26900</v>
       </c>
       <c r="G132">
@@ -9334,7 +9338,7 @@
       <c r="E133" t="s">
         <v>85</v>
       </c>
-      <c r="F133">
+      <c r="F133" s="14">
         <v>26900</v>
       </c>
       <c r="G133">
@@ -9375,7 +9379,7 @@
       <c r="E134" t="s">
         <v>69</v>
       </c>
-      <c r="F134">
+      <c r="F134" s="14">
         <v>29800</v>
       </c>
       <c r="G134">
@@ -9416,7 +9420,7 @@
       <c r="E135" t="s">
         <v>77</v>
       </c>
-      <c r="F135">
+      <c r="F135" s="14">
         <v>29800</v>
       </c>
       <c r="G135">
@@ -9457,7 +9461,7 @@
       <c r="E136" t="s">
         <v>79</v>
       </c>
-      <c r="F136">
+      <c r="F136" s="14">
         <v>29800</v>
       </c>
       <c r="G136">
@@ -9498,7 +9502,7 @@
       <c r="E137" t="s">
         <v>81</v>
       </c>
-      <c r="F137">
+      <c r="F137" s="14">
         <v>29800</v>
       </c>
       <c r="G137">
@@ -9539,7 +9543,7 @@
       <c r="E138" t="s">
         <v>83</v>
       </c>
-      <c r="F138">
+      <c r="F138" s="14">
         <v>29800</v>
       </c>
       <c r="G138">
@@ -9580,7 +9584,7 @@
       <c r="E139" t="s">
         <v>85</v>
       </c>
-      <c r="F139">
+      <c r="F139" s="14">
         <v>29800</v>
       </c>
       <c r="G139">
@@ -9621,7 +9625,7 @@
       <c r="E140" t="s">
         <v>69</v>
       </c>
-      <c r="F140">
+      <c r="F140" s="14">
         <v>31500</v>
       </c>
       <c r="G140">
@@ -9662,7 +9666,7 @@
       <c r="E141" t="s">
         <v>77</v>
       </c>
-      <c r="F141">
+      <c r="F141" s="14">
         <v>31500</v>
       </c>
       <c r="G141">
@@ -9703,7 +9707,7 @@
       <c r="E142" t="s">
         <v>79</v>
       </c>
-      <c r="F142">
+      <c r="F142" s="14">
         <v>31500</v>
       </c>
       <c r="G142">
@@ -9744,7 +9748,7 @@
       <c r="E143" t="s">
         <v>81</v>
       </c>
-      <c r="F143">
+      <c r="F143" s="14">
         <v>31500</v>
       </c>
       <c r="G143">
@@ -9785,7 +9789,7 @@
       <c r="E144" t="s">
         <v>83</v>
       </c>
-      <c r="F144">
+      <c r="F144" s="14">
         <v>31500</v>
       </c>
       <c r="G144">
@@ -9826,7 +9830,7 @@
       <c r="E145" t="s">
         <v>85</v>
       </c>
-      <c r="F145">
+      <c r="F145" s="14">
         <v>31500</v>
       </c>
       <c r="G145">
@@ -9867,7 +9871,7 @@
       <c r="E146" t="s">
         <v>69</v>
       </c>
-      <c r="F146">
+      <c r="F146" s="14">
         <v>31500</v>
       </c>
       <c r="G146">
@@ -9905,7 +9909,7 @@
       <c r="E147" t="s">
         <v>77</v>
       </c>
-      <c r="F147">
+      <c r="F147" s="14">
         <v>31500</v>
       </c>
       <c r="G147">
@@ -9943,7 +9947,7 @@
       <c r="E148" t="s">
         <v>79</v>
       </c>
-      <c r="F148">
+      <c r="F148" s="14">
         <v>31500</v>
       </c>
       <c r="G148">
@@ -9981,7 +9985,7 @@
       <c r="E149" t="s">
         <v>81</v>
       </c>
-      <c r="F149">
+      <c r="F149" s="14">
         <v>31500</v>
       </c>
       <c r="G149">
@@ -10019,7 +10023,7 @@
       <c r="E150" t="s">
         <v>83</v>
       </c>
-      <c r="F150">
+      <c r="F150" s="14">
         <v>31500</v>
       </c>
       <c r="G150">
@@ -10057,7 +10061,7 @@
       <c r="E151" t="s">
         <v>85</v>
       </c>
-      <c r="F151">
+      <c r="F151" s="14">
         <v>31500</v>
       </c>
       <c r="G151">

</xml_diff>